<commit_message>
Fight card : Ethan Bégué (SHO) contre Ethan Icaze (FAK) en exhibition
Les deux exhibitions sans adversaire n'en font plus qu'une, entre deux clubs.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BG94EkAj2aYi3kCmvbMWy9
</commit_message>
<xml_diff>
--- a/dojo/interclub/shidokan-challenge-974-fight-card.xlsx
+++ b/dojo/interclub/shidokan-challenge-974-fight-card.xlsx
@@ -16,7 +16,7 @@
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Combattants!$A$1:$M$46</definedName>
     <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Titles" vbProcedure="false">'Fight card'!$5:$5</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Fight card'!$A$5:$R$46</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Fight card'!$A$5:$R$45</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="720" uniqueCount="264">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="711" uniqueCount="263">
   <si>
     <t xml:space="preserve">SHIDOKAN CHALLENGE 974 — ORDRE DES COMBATS</t>
   </si>
@@ -298,34 +298,31 @@
     <t xml:space="preserve">09h52</t>
   </si>
   <si>
-    <t xml:space="preserve">Benjamin lourd</t>
+    <t xml:space="preserve">Benjamin lourd / Cadet</t>
   </si>
   <si>
     <t xml:space="preserve">Ethan BÉGUÉ</t>
   </si>
   <si>
+    <t xml:space="preserve">Ethan ICAZE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">09h56</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eden PRUDENT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Boxing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shidoboxing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chloé FONTAINE</t>
+  </si>
+  <si>
     <t xml:space="preserve">Adversaire à définir</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cadet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ethan ICAZE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">09h56</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Eden PRUDENT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Boxing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Shidoboxing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chloé FONTAINE</t>
   </si>
   <si>
     <t xml:space="preserve">10h00</t>
@@ -1573,7 +1570,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:R46"/>
+  <dimension ref="A1:R45"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -1605,7 +1602,7 @@
       </c>
       <c r="O1" s="3" t="n">
         <f aca="false">COUNTA(I6:I200)</f>
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1629,7 +1626,7 @@
       </c>
       <c r="O3" s="3" t="n">
         <f aca="false">O1-O2</f>
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2536,12 +2533,12 @@
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(I22,Combattants!$A$2:$A$200,0)),"")</f>
         <v>SHO</v>
       </c>
-      <c r="K22" s="15" t="s">
+      <c r="K22" s="14" t="s">
         <v>80</v>
       </c>
       <c r="L22" s="13" t="str">
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(K22,Combattants!$A$2:$A$200,0)),"")</f>
-        <v/>
+        <v>FAK</v>
       </c>
       <c r="M22" s="9" t="s">
         <v>31</v>
@@ -2557,22 +2554,22 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="9" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="C23" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D23" s="10" t="s">
         <v>24</v>
       </c>
       <c r="E23" s="11" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="F23" s="10" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="G23" s="10" t="s">
         <v>27</v>
@@ -2585,14 +2582,14 @@
       </c>
       <c r="J23" s="13" t="str">
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(I23,Combattants!$A$2:$A$200,0)),"")</f>
-        <v>FAK</v>
-      </c>
-      <c r="K23" s="15" t="s">
-        <v>80</v>
+        <v>FUK</v>
+      </c>
+      <c r="K23" s="14" t="s">
+        <v>76</v>
       </c>
       <c r="L23" s="13" t="str">
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(K23,Combattants!$A$2:$A$200,0)),"")</f>
-        <v/>
+        <v>SHO</v>
       </c>
       <c r="M23" s="9" t="s">
         <v>31</v>
@@ -2608,42 +2605,42 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="9" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C24" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D24" s="10" t="s">
         <v>24</v>
       </c>
       <c r="E24" s="11" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="F24" s="10" t="s">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="G24" s="10" t="s">
-        <v>27</v>
+        <v>84</v>
       </c>
       <c r="H24" s="10" t="s">
         <v>28</v>
       </c>
       <c r="I24" s="12" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="J24" s="13" t="str">
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(I24,Combattants!$A$2:$A$200,0)),"")</f>
-        <v>FUK</v>
-      </c>
-      <c r="K24" s="14" t="s">
-        <v>76</v>
+        <v>SHO</v>
+      </c>
+      <c r="K24" s="15" t="s">
+        <v>86</v>
       </c>
       <c r="L24" s="13" t="str">
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(K24,Combattants!$A$2:$A$200,0)),"")</f>
-        <v>SHO</v>
+        <v/>
       </c>
       <c r="M24" s="9" t="s">
         <v>31</v>
@@ -2659,38 +2656,38 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="9" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="C25" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D25" s="10" t="s">
         <v>24</v>
       </c>
       <c r="E25" s="11" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="F25" s="10" t="s">
         <v>41</v>
       </c>
       <c r="G25" s="10" t="s">
-        <v>86</v>
+        <v>27</v>
       </c>
       <c r="H25" s="10" t="s">
         <v>28</v>
       </c>
       <c r="I25" s="12" t="s">
-        <v>87</v>
+        <v>39</v>
       </c>
       <c r="J25" s="13" t="str">
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(I25,Combattants!$A$2:$A$200,0)),"")</f>
-        <v>SHO</v>
+        <v>FAK</v>
       </c>
       <c r="K25" s="15" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="L25" s="13" t="str">
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(K25,Combattants!$A$2:$A$200,0)),"")</f>
@@ -2710,22 +2707,22 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="9" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C26" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D26" s="10" t="s">
         <v>24</v>
       </c>
       <c r="E26" s="11" t="s">
-        <v>89</v>
+        <v>46</v>
       </c>
       <c r="F26" s="10" t="s">
-        <v>41</v>
+        <v>64</v>
       </c>
       <c r="G26" s="10" t="s">
         <v>27</v>
@@ -2733,15 +2730,15 @@
       <c r="H26" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="I26" s="12" t="s">
-        <v>39</v>
+      <c r="I26" s="16" t="s">
+        <v>89</v>
       </c>
       <c r="J26" s="13" t="str">
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(I26,Combattants!$A$2:$A$200,0)),"")</f>
-        <v>FAK</v>
+        <v/>
       </c>
       <c r="K26" s="15" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="L26" s="13" t="str">
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(K26,Combattants!$A$2:$A$200,0)),"")</f>
@@ -2761,22 +2758,22 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="9" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="C27" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D27" s="10" t="s">
         <v>24</v>
       </c>
       <c r="E27" s="11" t="s">
-        <v>46</v>
+        <v>74</v>
       </c>
       <c r="F27" s="10" t="s">
-        <v>64</v>
+        <v>26</v>
       </c>
       <c r="G27" s="10" t="s">
         <v>27</v>
@@ -2784,19 +2781,19 @@
       <c r="H27" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="I27" s="16" t="s">
-        <v>90</v>
+      <c r="I27" s="12" t="s">
+        <v>75</v>
       </c>
       <c r="J27" s="13" t="str">
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(I27,Combattants!$A$2:$A$200,0)),"")</f>
-        <v/>
-      </c>
-      <c r="K27" s="15" t="s">
-        <v>91</v>
+        <v>FUK</v>
+      </c>
+      <c r="K27" s="14" t="s">
+        <v>82</v>
       </c>
       <c r="L27" s="13" t="str">
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(K27,Combattants!$A$2:$A$200,0)),"")</f>
-        <v/>
+        <v>FUK</v>
       </c>
       <c r="M27" s="9" t="s">
         <v>31</v>
@@ -2812,22 +2809,22 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="9" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C28" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D28" s="10" t="s">
         <v>24</v>
       </c>
       <c r="E28" s="11" t="s">
-        <v>74</v>
+        <v>46</v>
       </c>
       <c r="F28" s="10" t="s">
-        <v>26</v>
+        <v>67</v>
       </c>
       <c r="G28" s="10" t="s">
         <v>27</v>
@@ -2835,19 +2832,19 @@
       <c r="H28" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="I28" s="12" t="s">
-        <v>75</v>
+      <c r="I28" s="16" t="s">
+        <v>92</v>
       </c>
       <c r="J28" s="13" t="str">
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(I28,Combattants!$A$2:$A$200,0)),"")</f>
-        <v>FUK</v>
-      </c>
-      <c r="K28" s="14" t="s">
-        <v>84</v>
+        <v/>
+      </c>
+      <c r="K28" s="15" t="s">
+        <v>93</v>
       </c>
       <c r="L28" s="13" t="str">
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(K28,Combattants!$A$2:$A$200,0)),"")</f>
-        <v>FUK</v>
+        <v/>
       </c>
       <c r="M28" s="9" t="s">
         <v>31</v>
@@ -2863,22 +2860,22 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="9" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C29" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D29" s="10" t="s">
         <v>24</v>
       </c>
       <c r="E29" s="11" t="s">
-        <v>46</v>
+        <v>63</v>
       </c>
       <c r="F29" s="10" t="s">
-        <v>67</v>
+        <v>95</v>
       </c>
       <c r="G29" s="10" t="s">
         <v>27</v>
@@ -2887,14 +2884,14 @@
         <v>28</v>
       </c>
       <c r="I29" s="16" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="J29" s="13" t="str">
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(I29,Combattants!$A$2:$A$200,0)),"")</f>
         <v/>
       </c>
       <c r="K29" s="15" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="L29" s="13" t="str">
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(K29,Combattants!$A$2:$A$200,0)),"")</f>
@@ -2914,13 +2911,13 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="9" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C30" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D30" s="10" t="s">
         <v>24</v>
@@ -2929,7 +2926,7 @@
         <v>63</v>
       </c>
       <c r="F30" s="10" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="G30" s="10" t="s">
         <v>27</v>
@@ -2938,14 +2935,14 @@
         <v>28</v>
       </c>
       <c r="I30" s="16" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="J30" s="13" t="str">
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(I30,Combattants!$A$2:$A$200,0)),"")</f>
         <v/>
       </c>
       <c r="K30" s="15" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="L30" s="13" t="str">
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(K30,Combattants!$A$2:$A$200,0)),"")</f>
@@ -2965,22 +2962,22 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="9" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B31" s="9" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="C31" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D31" s="10" t="s">
         <v>24</v>
       </c>
       <c r="E31" s="11" t="s">
-        <v>63</v>
+        <v>46</v>
       </c>
       <c r="F31" s="10" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="G31" s="10" t="s">
         <v>27</v>
@@ -2989,14 +2986,14 @@
         <v>28</v>
       </c>
       <c r="I31" s="16" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="J31" s="13" t="str">
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(I31,Combattants!$A$2:$A$200,0)),"")</f>
         <v/>
       </c>
       <c r="K31" s="15" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="L31" s="13" t="str">
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(K31,Combattants!$A$2:$A$200,0)),"")</f>
@@ -3016,13 +3013,13 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="9" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C32" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D32" s="10" t="s">
         <v>24</v>
@@ -3031,7 +3028,7 @@
         <v>46</v>
       </c>
       <c r="F32" s="10" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="G32" s="10" t="s">
         <v>27</v>
@@ -3040,14 +3037,14 @@
         <v>28</v>
       </c>
       <c r="I32" s="16" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="J32" s="13" t="str">
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(I32,Combattants!$A$2:$A$200,0)),"")</f>
         <v/>
       </c>
       <c r="K32" s="15" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="L32" s="13" t="str">
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(K32,Combattants!$A$2:$A$200,0)),"")</f>
@@ -3067,42 +3064,42 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="9" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="C33" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D33" s="10" t="s">
-        <v>24</v>
+        <v>107</v>
       </c>
       <c r="E33" s="11" t="s">
-        <v>46</v>
+        <v>108</v>
       </c>
       <c r="F33" s="10" t="s">
-        <v>99</v>
+        <v>37</v>
       </c>
       <c r="G33" s="10" t="s">
         <v>27</v>
       </c>
       <c r="H33" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="I33" s="16" t="s">
-        <v>105</v>
+        <v>109</v>
+      </c>
+      <c r="I33" s="12" t="s">
+        <v>110</v>
       </c>
       <c r="J33" s="13" t="str">
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(I33,Combattants!$A$2:$A$200,0)),"")</f>
-        <v/>
-      </c>
-      <c r="K33" s="15" t="s">
-        <v>106</v>
+        <v>SHO</v>
+      </c>
+      <c r="K33" s="14" t="s">
+        <v>111</v>
       </c>
       <c r="L33" s="13" t="str">
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(K33,Combattants!$A$2:$A$200,0)),"")</f>
-        <v/>
+        <v>SHO</v>
       </c>
       <c r="M33" s="9" t="s">
         <v>31</v>
@@ -3118,38 +3115,38 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="9" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B34" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="C34" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D34" s="10" t="s">
         <v>107</v>
       </c>
-      <c r="C34" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="D34" s="10" t="s">
-        <v>108</v>
-      </c>
       <c r="E34" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="F34" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G34" s="10" t="s">
+        <v>113</v>
+      </c>
+      <c r="H34" s="10" t="s">
         <v>109</v>
       </c>
-      <c r="F34" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="G34" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="H34" s="10" t="s">
-        <v>110</v>
-      </c>
       <c r="I34" s="12" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="J34" s="13" t="str">
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(I34,Combattants!$A$2:$A$200,0)),"")</f>
         <v>SHO</v>
       </c>
       <c r="K34" s="14" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="L34" s="13" t="str">
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(K34,Combattants!$A$2:$A$200,0)),"")</f>
@@ -3169,42 +3166,42 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="9" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B35" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="C35" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" s="10" t="s">
         <v>107</v>
       </c>
-      <c r="C35" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="D35" s="10" t="s">
-        <v>108</v>
-      </c>
       <c r="E35" s="11" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="F35" s="10" t="s">
-        <v>26</v>
+        <v>64</v>
       </c>
       <c r="G35" s="10" t="s">
-        <v>114</v>
+        <v>27</v>
       </c>
       <c r="H35" s="10" t="s">
-        <v>110</v>
-      </c>
-      <c r="I35" s="12" t="s">
-        <v>115</v>
+        <v>109</v>
+      </c>
+      <c r="I35" s="16" t="s">
+        <v>118</v>
       </c>
       <c r="J35" s="13" t="str">
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(I35,Combattants!$A$2:$A$200,0)),"")</f>
-        <v>SHO</v>
-      </c>
-      <c r="K35" s="14" t="s">
-        <v>116</v>
+        <v/>
+      </c>
+      <c r="K35" s="15" t="s">
+        <v>118</v>
       </c>
       <c r="L35" s="13" t="str">
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(K35,Combattants!$A$2:$A$200,0)),"")</f>
-        <v>SHO</v>
+        <v/>
       </c>
       <c r="M35" s="9" t="s">
         <v>31</v>
@@ -3220,38 +3217,38 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="9" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B36" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="C36" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D36" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="E36" s="11" t="s">
         <v>117</v>
       </c>
-      <c r="C36" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="D36" s="10" t="s">
-        <v>108</v>
-      </c>
-      <c r="E36" s="11" t="s">
+      <c r="F36" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="G36" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="H36" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="I36" s="16" t="s">
         <v>118</v>
-      </c>
-      <c r="F36" s="10" t="s">
-        <v>64</v>
-      </c>
-      <c r="G36" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="H36" s="10" t="s">
-        <v>110</v>
-      </c>
-      <c r="I36" s="16" t="s">
-        <v>119</v>
       </c>
       <c r="J36" s="13" t="str">
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(I36,Combattants!$A$2:$A$200,0)),"")</f>
         <v/>
       </c>
       <c r="K36" s="15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="L36" s="13" t="str">
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(K36,Combattants!$A$2:$A$200,0)),"")</f>
@@ -3271,38 +3268,38 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="9" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B37" s="9" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C37" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D37" s="10" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E37" s="11" t="s">
+        <v>120</v>
+      </c>
+      <c r="F37" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="G37" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="H37" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="I37" s="16" t="s">
         <v>118</v>
-      </c>
-      <c r="F37" s="10" t="s">
-        <v>67</v>
-      </c>
-      <c r="G37" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="H37" s="10" t="s">
-        <v>110</v>
-      </c>
-      <c r="I37" s="16" t="s">
-        <v>119</v>
       </c>
       <c r="J37" s="13" t="str">
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(I37,Combattants!$A$2:$A$200,0)),"")</f>
         <v/>
       </c>
       <c r="K37" s="15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="L37" s="13" t="str">
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(K37,Combattants!$A$2:$A$200,0)),"")</f>
@@ -3322,42 +3319,42 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="9" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B38" s="9" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C38" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D38" s="10" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E38" s="11" t="s">
-        <v>121</v>
+        <v>112</v>
       </c>
       <c r="F38" s="10" t="s">
-        <v>122</v>
+        <v>26</v>
       </c>
       <c r="G38" s="10" t="s">
-        <v>27</v>
+        <v>113</v>
       </c>
       <c r="H38" s="10" t="s">
-        <v>110</v>
-      </c>
-      <c r="I38" s="16" t="s">
-        <v>119</v>
+        <v>109</v>
+      </c>
+      <c r="I38" s="12" t="s">
+        <v>114</v>
       </c>
       <c r="J38" s="13" t="str">
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(I38,Combattants!$A$2:$A$200,0)),"")</f>
-        <v/>
-      </c>
-      <c r="K38" s="15" t="s">
-        <v>119</v>
+        <v>SHO</v>
+      </c>
+      <c r="K38" s="14" t="s">
+        <v>122</v>
       </c>
       <c r="L38" s="13" t="str">
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(K38,Combattants!$A$2:$A$200,0)),"")</f>
-        <v/>
+        <v>SHO</v>
       </c>
       <c r="M38" s="9" t="s">
         <v>31</v>
@@ -3373,42 +3370,42 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="9" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="C39" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D39" s="10" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E39" s="11" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="F39" s="10" t="s">
-        <v>26</v>
+        <v>95</v>
       </c>
       <c r="G39" s="10" t="s">
-        <v>114</v>
+        <v>27</v>
       </c>
       <c r="H39" s="10" t="s">
-        <v>110</v>
-      </c>
-      <c r="I39" s="12" t="s">
-        <v>115</v>
+        <v>109</v>
+      </c>
+      <c r="I39" s="16" t="s">
+        <v>124</v>
       </c>
       <c r="J39" s="13" t="str">
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(I39,Combattants!$A$2:$A$200,0)),"")</f>
-        <v>SHO</v>
-      </c>
-      <c r="K39" s="14" t="s">
-        <v>123</v>
+        <v/>
+      </c>
+      <c r="K39" s="15" t="s">
+        <v>125</v>
       </c>
       <c r="L39" s="13" t="str">
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(K39,Combattants!$A$2:$A$200,0)),"")</f>
-        <v>SHO</v>
+        <v/>
       </c>
       <c r="M39" s="9" t="s">
         <v>31</v>
@@ -3424,38 +3421,38 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="9" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B40" s="9" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C40" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D40" s="10" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E40" s="11" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F40" s="10" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="G40" s="10" t="s">
         <v>27</v>
       </c>
       <c r="H40" s="10" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="I40" s="16" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="J40" s="13" t="str">
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(I40,Combattants!$A$2:$A$200,0)),"")</f>
         <v/>
       </c>
       <c r="K40" s="15" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="L40" s="13" t="str">
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(K40,Combattants!$A$2:$A$200,0)),"")</f>
@@ -3471,42 +3468,44 @@
       </c>
       <c r="P40" s="9"/>
       <c r="Q40" s="9"/>
-      <c r="R40" s="11"/>
+      <c r="R40" s="11" t="s">
+        <v>128</v>
+      </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="9" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B41" s="9" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="C41" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D41" s="10" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E41" s="11" t="s">
+        <v>120</v>
+      </c>
+      <c r="F41" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="G41" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="H41" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="I41" s="16" t="s">
         <v>118</v>
-      </c>
-      <c r="F41" s="10" t="s">
-        <v>99</v>
-      </c>
-      <c r="G41" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="H41" s="10" t="s">
-        <v>110</v>
-      </c>
-      <c r="I41" s="16" t="s">
-        <v>127</v>
       </c>
       <c r="J41" s="13" t="str">
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(I41,Combattants!$A$2:$A$200,0)),"")</f>
         <v/>
       </c>
       <c r="K41" s="15" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="L41" s="13" t="str">
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(K41,Combattants!$A$2:$A$200,0)),"")</f>
@@ -3522,44 +3521,42 @@
       </c>
       <c r="P41" s="9"/>
       <c r="Q41" s="9"/>
-      <c r="R41" s="11" t="s">
-        <v>129</v>
-      </c>
+      <c r="R41" s="11"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="9" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B42" s="9" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C42" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D42" s="10" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E42" s="11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F42" s="10" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="G42" s="10" t="s">
         <v>27</v>
       </c>
       <c r="H42" s="10" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="I42" s="16" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="J42" s="13" t="str">
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(I42,Combattants!$A$2:$A$200,0)),"")</f>
         <v/>
       </c>
       <c r="K42" s="15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="L42" s="13" t="str">
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(K42,Combattants!$A$2:$A$200,0)),"")</f>
@@ -3579,42 +3576,42 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="9" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B43" s="9" t="s">
         <v>130</v>
       </c>
       <c r="C43" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D43" s="10" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E43" s="11" t="s">
-        <v>121</v>
+        <v>112</v>
       </c>
       <c r="F43" s="10" t="s">
-        <v>67</v>
+        <v>26</v>
       </c>
       <c r="G43" s="10" t="s">
-        <v>27</v>
+        <v>113</v>
       </c>
       <c r="H43" s="10" t="s">
-        <v>110</v>
-      </c>
-      <c r="I43" s="16" t="s">
-        <v>119</v>
+        <v>109</v>
+      </c>
+      <c r="I43" s="12" t="s">
+        <v>115</v>
       </c>
       <c r="J43" s="13" t="str">
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(I43,Combattants!$A$2:$A$200,0)),"")</f>
-        <v/>
-      </c>
-      <c r="K43" s="15" t="s">
-        <v>119</v>
+        <v>SHO</v>
+      </c>
+      <c r="K43" s="14" t="s">
+        <v>122</v>
       </c>
       <c r="L43" s="13" t="str">
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(K43,Combattants!$A$2:$A$200,0)),"")</f>
-        <v/>
+        <v>SHO</v>
       </c>
       <c r="M43" s="9" t="s">
         <v>31</v>
@@ -3630,7 +3627,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="9" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B44" s="9" t="s">
         <v>131</v>
@@ -3639,33 +3636,33 @@
         <v>1</v>
       </c>
       <c r="D44" s="10" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E44" s="11" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="F44" s="10" t="s">
-        <v>26</v>
+        <v>95</v>
       </c>
       <c r="G44" s="10" t="s">
-        <v>114</v>
+        <v>27</v>
       </c>
       <c r="H44" s="10" t="s">
-        <v>110</v>
-      </c>
-      <c r="I44" s="12" t="s">
-        <v>116</v>
+        <v>109</v>
+      </c>
+      <c r="I44" s="16" t="s">
+        <v>132</v>
       </c>
       <c r="J44" s="13" t="str">
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(I44,Combattants!$A$2:$A$200,0)),"")</f>
-        <v>SHO</v>
-      </c>
-      <c r="K44" s="14" t="s">
-        <v>123</v>
+        <v/>
+      </c>
+      <c r="K44" s="15" t="s">
+        <v>133</v>
       </c>
       <c r="L44" s="13" t="str">
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(K44,Combattants!$A$2:$A$200,0)),"")</f>
-        <v>SHO</v>
+        <v/>
       </c>
       <c r="M44" s="9" t="s">
         <v>31</v>
@@ -3681,38 +3678,38 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="9" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B45" s="9" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C45" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D45" s="10" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E45" s="11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F45" s="10" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="G45" s="10" t="s">
         <v>27</v>
       </c>
       <c r="H45" s="10" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="I45" s="16" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="J45" s="13" t="str">
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(I45,Combattants!$A$2:$A$200,0)),"")</f>
         <v/>
       </c>
       <c r="K45" s="15" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="L45" s="13" t="str">
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(K45,Combattants!$A$2:$A$200,0)),"")</f>
@@ -3728,63 +3725,12 @@
       </c>
       <c r="P45" s="9"/>
       <c r="Q45" s="9"/>
-      <c r="R45" s="11"/>
-    </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="9" t="n">
-        <v>41</v>
-      </c>
-      <c r="B46" s="9" t="s">
-        <v>132</v>
-      </c>
-      <c r="C46" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="D46" s="10" t="s">
-        <v>108</v>
-      </c>
-      <c r="E46" s="11" t="s">
-        <v>121</v>
-      </c>
-      <c r="F46" s="10" t="s">
-        <v>99</v>
-      </c>
-      <c r="G46" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="H46" s="10" t="s">
-        <v>110</v>
-      </c>
-      <c r="I46" s="16" t="s">
-        <v>135</v>
-      </c>
-      <c r="J46" s="13" t="str">
-        <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(I46,Combattants!$A$2:$A$200,0)),"")</f>
-        <v/>
-      </c>
-      <c r="K46" s="15" t="s">
+      <c r="R45" s="11" t="s">
         <v>136</v>
       </c>
-      <c r="L46" s="13" t="str">
-        <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(K46,Combattants!$A$2:$A$200,0)),"")</f>
-        <v/>
-      </c>
-      <c r="M46" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="N46" s="9"/>
-      <c r="O46" s="13" t="str">
-        <f aca="false">IF(N46="Rouge",I46,IF(N46="Bleu",K46,IF(N46="Nul","Match nul","")))</f>
-        <v/>
-      </c>
-      <c r="P46" s="9"/>
-      <c r="Q46" s="9"/>
-      <c r="R46" s="11" t="s">
-        <v>137</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:R46"/>
+  <autoFilter ref="A5:R45"/>
   <conditionalFormatting sqref="A6:R200">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
       <formula>$M6="Terminé"</formula>
@@ -3860,47 +3806,47 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="17" t="s">
+        <v>137</v>
+      </c>
+      <c r="B1" s="18" t="s">
         <v>138</v>
-      </c>
-      <c r="B1" s="18" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="17" t="s">
+        <v>139</v>
+      </c>
+      <c r="B2" s="18" t="s">
         <v>140</v>
-      </c>
-      <c r="B2" s="18" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="17" t="s">
+        <v>141</v>
+      </c>
+      <c r="B3" s="18" t="s">
         <v>142</v>
-      </c>
-      <c r="B3" s="18" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="17" t="s">
+        <v>143</v>
+      </c>
+      <c r="B4" s="18" t="s">
         <v>144</v>
-      </c>
-      <c r="B4" s="18" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="17" t="s">
+        <v>145</v>
+      </c>
+      <c r="B5" s="18" t="s">
         <v>146</v>
-      </c>
-      <c r="B5" s="18" t="s">
-        <v>147</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="17" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B6" s="18" t="n">
         <v>2</v>
@@ -3908,10 +3854,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="17" t="s">
+        <v>148</v>
+      </c>
+      <c r="B7" s="18" t="s">
         <v>149</v>
-      </c>
-      <c r="B7" s="18" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3919,60 +3865,60 @@
         <v>7</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="20" t="s">
+        <v>151</v>
+      </c>
+      <c r="B10" s="20" t="s">
         <v>152</v>
-      </c>
-      <c r="B10" s="20" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="s">
+        <v>153</v>
+      </c>
+      <c r="B11" s="20" t="s">
         <v>154</v>
-      </c>
-      <c r="B11" s="20" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="20" t="s">
+        <v>155</v>
+      </c>
+      <c r="B12" s="20" t="s">
         <v>156</v>
-      </c>
-      <c r="B12" s="20" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="20" t="s">
+        <v>157</v>
+      </c>
+      <c r="B13" s="20" t="s">
         <v>158</v>
-      </c>
-      <c r="B13" s="20" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="20" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B14" s="20" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="20" t="s">
+        <v>160</v>
+      </c>
+      <c r="B15" s="20" t="s">
         <v>161</v>
-      </c>
-      <c r="B15" s="20" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
   </sheetData>
@@ -4009,40 +3955,40 @@
   <sheetData>
     <row r="1" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="B1" s="6" t="s">
         <v>164</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="C1" s="6" t="s">
         <v>165</v>
-      </c>
-      <c r="C1" s="6" t="s">
-        <v>166</v>
       </c>
       <c r="D1" s="6" t="s">
         <v>15</v>
       </c>
       <c r="E1" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="F1" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="G1" s="6" t="s">
         <v>168</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="H1" s="6" t="s">
         <v>169</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="I1" s="6" t="s">
         <v>170</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="J1" s="6" t="s">
         <v>171</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="K1" s="6" t="s">
         <v>172</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="L1" s="6" t="s">
         <v>173</v>
-      </c>
-      <c r="L1" s="6" t="s">
-        <v>174</v>
       </c>
       <c r="M1" s="6" t="s">
         <v>22</v>
@@ -4054,23 +4000,23 @@
         <v>Ethan ICAZE</v>
       </c>
       <c r="B2" s="20" t="s">
+        <v>174</v>
+      </c>
+      <c r="C2" s="20" t="s">
         <v>175</v>
       </c>
-      <c r="C2" s="20" t="s">
-        <v>176</v>
-      </c>
       <c r="D2" s="20" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E2" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D2,Clubs!$A$2:$A$20,0)),"")</f>
         <v>FAK</v>
       </c>
       <c r="F2" s="20" t="s">
+        <v>176</v>
+      </c>
+      <c r="G2" s="20" t="s">
         <v>177</v>
-      </c>
-      <c r="G2" s="20" t="s">
-        <v>178</v>
       </c>
       <c r="H2" s="20"/>
       <c r="I2" s="20"/>
@@ -4090,20 +4036,20 @@
         <v>Lorentz PAYET</v>
       </c>
       <c r="B3" s="20" t="s">
+        <v>178</v>
+      </c>
+      <c r="C3" s="20" t="s">
         <v>179</v>
       </c>
-      <c r="C3" s="20" t="s">
-        <v>180</v>
-      </c>
       <c r="D3" s="20" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E3" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D3,Clubs!$A$2:$A$20,0)),"")</f>
         <v>FAK</v>
       </c>
       <c r="F3" s="20" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G3" s="20" t="s">
         <v>46</v>
@@ -4128,23 +4074,23 @@
         <v>Melina FOLIO</v>
       </c>
       <c r="B4" s="20" t="s">
+        <v>180</v>
+      </c>
+      <c r="C4" s="20" t="s">
         <v>181</v>
       </c>
-      <c r="C4" s="20" t="s">
-        <v>182</v>
-      </c>
       <c r="D4" s="20" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E4" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D4,Clubs!$A$2:$A$20,0)),"")</f>
         <v>FAK</v>
       </c>
       <c r="F4" s="20" t="s">
+        <v>182</v>
+      </c>
+      <c r="G4" s="20" t="s">
         <v>183</v>
-      </c>
-      <c r="G4" s="20" t="s">
-        <v>184</v>
       </c>
       <c r="H4" s="20"/>
       <c r="I4" s="20" t="n">
@@ -4159,7 +4105,7 @@
         <v>2</v>
       </c>
       <c r="M4" s="20" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4168,29 +4114,29 @@
         <v>Mike</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C5" s="20"/>
       <c r="D5" s="20" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E5" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D5,Clubs!$A$2:$A$20,0)),"")</f>
         <v>FAK</v>
       </c>
       <c r="F5" s="20" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G5" s="20" t="s">
+        <v>186</v>
+      </c>
+      <c r="H5" s="20" t="s">
         <v>187</v>
-      </c>
-      <c r="H5" s="20" t="s">
-        <v>188</v>
       </c>
       <c r="I5" s="20"/>
       <c r="J5" s="20"/>
       <c r="K5" s="20" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="L5" s="22" t="n">
         <f aca="false">COUNTIF('Fight card'!$I$6:$I$200,A5)+COUNTIF('Fight card'!$K$6:$K$200,A5)</f>
@@ -4204,20 +4150,20 @@
         <v>Raphaël FRAYNAL</v>
       </c>
       <c r="B6" s="20" t="s">
+        <v>188</v>
+      </c>
+      <c r="C6" s="20" t="s">
         <v>189</v>
       </c>
-      <c r="C6" s="20" t="s">
-        <v>190</v>
-      </c>
       <c r="D6" s="20" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E6" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D6,Clubs!$A$2:$A$20,0)),"")</f>
         <v>FAK</v>
       </c>
       <c r="F6" s="20" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G6" s="20" t="s">
         <v>46</v>
@@ -4242,23 +4188,23 @@
         <v>Basile ABEL</v>
       </c>
       <c r="B7" s="20" t="s">
+        <v>190</v>
+      </c>
+      <c r="C7" s="20" t="s">
         <v>191</v>
       </c>
-      <c r="C7" s="20" t="s">
+      <c r="D7" s="20" t="s">
         <v>192</v>
-      </c>
-      <c r="D7" s="20" t="s">
-        <v>193</v>
       </c>
       <c r="E7" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D7,Clubs!$A$2:$A$20,0)),"")</f>
         <v>FUK</v>
       </c>
       <c r="F7" s="20" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G7" s="20" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="H7" s="20"/>
       <c r="I7" s="20"/>
@@ -4278,20 +4224,20 @@
         <v>Benjamin LEGRAND</v>
       </c>
       <c r="B8" s="20" t="s">
+        <v>193</v>
+      </c>
+      <c r="C8" s="20" t="s">
         <v>194</v>
       </c>
-      <c r="C8" s="20" t="s">
-        <v>195</v>
-      </c>
       <c r="D8" s="20" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E8" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D8,Clubs!$A$2:$A$20,0)),"")</f>
         <v>FUK</v>
       </c>
       <c r="F8" s="20" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G8" s="20" t="s">
         <v>46</v>
@@ -4314,23 +4260,23 @@
         <v>Bilal SALIMA</v>
       </c>
       <c r="B9" s="20" t="s">
+        <v>195</v>
+      </c>
+      <c r="C9" s="20" t="s">
         <v>196</v>
       </c>
-      <c r="C9" s="20" t="s">
-        <v>197</v>
-      </c>
       <c r="D9" s="20" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E9" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D9,Clubs!$A$2:$A$20,0)),"")</f>
         <v>FUK</v>
       </c>
       <c r="F9" s="20" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G9" s="20" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="H9" s="20"/>
       <c r="I9" s="20"/>
@@ -4350,20 +4296,20 @@
         <v>Camilya BACAR</v>
       </c>
       <c r="B10" s="20" t="s">
+        <v>198</v>
+      </c>
+      <c r="C10" s="20" t="s">
         <v>199</v>
       </c>
-      <c r="C10" s="20" t="s">
-        <v>200</v>
-      </c>
       <c r="D10" s="20" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E10" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D10,Clubs!$A$2:$A$20,0)),"")</f>
         <v>FUK</v>
       </c>
       <c r="F10" s="20" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G10" s="20" t="s">
         <v>25</v>
@@ -4386,23 +4332,23 @@
         <v>Clément DELMAS</v>
       </c>
       <c r="B11" s="20" t="s">
+        <v>200</v>
+      </c>
+      <c r="C11" s="20" t="s">
         <v>201</v>
       </c>
-      <c r="C11" s="20" t="s">
-        <v>202</v>
-      </c>
       <c r="D11" s="20" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E11" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D11,Clubs!$A$2:$A$20,0)),"")</f>
         <v>FUK</v>
       </c>
       <c r="F11" s="20" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G11" s="20" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="H11" s="20"/>
       <c r="I11" s="20"/>
@@ -4415,7 +4361,7 @@
         <v>0</v>
       </c>
       <c r="M11" s="20" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4424,20 +4370,20 @@
         <v>Eden BOYER</v>
       </c>
       <c r="B12" s="20" t="s">
+        <v>203</v>
+      </c>
+      <c r="C12" s="20" t="s">
         <v>204</v>
       </c>
-      <c r="C12" s="20" t="s">
-        <v>205</v>
-      </c>
       <c r="D12" s="20" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E12" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D12,Clubs!$A$2:$A$20,0)),"")</f>
         <v>FUK</v>
       </c>
       <c r="F12" s="20" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G12" s="20" t="s">
         <v>46</v>
@@ -4460,23 +4406,23 @@
         <v>Eden PRUDENT</v>
       </c>
       <c r="B13" s="20" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C13" s="20" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D13" s="20" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E13" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D13,Clubs!$A$2:$A$20,0)),"")</f>
         <v>FUK</v>
       </c>
       <c r="F13" s="20" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G13" s="20" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="H13" s="20"/>
       <c r="I13" s="20"/>
@@ -4496,23 +4442,23 @@
         <v>Elie-Rose THOMAS</v>
       </c>
       <c r="B14" s="20" t="s">
+        <v>206</v>
+      </c>
+      <c r="C14" s="20" t="s">
         <v>207</v>
       </c>
-      <c r="C14" s="20" t="s">
-        <v>208</v>
-      </c>
       <c r="D14" s="20" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E14" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D14,Clubs!$A$2:$A$20,0)),"")</f>
         <v>FUK</v>
       </c>
       <c r="F14" s="20" t="s">
+        <v>182</v>
+      </c>
+      <c r="G14" s="20" t="s">
         <v>183</v>
-      </c>
-      <c r="G14" s="20" t="s">
-        <v>184</v>
       </c>
       <c r="H14" s="20"/>
       <c r="I14" s="20"/>
@@ -4532,23 +4478,23 @@
         <v>Ella GRUCHET</v>
       </c>
       <c r="B15" s="20" t="s">
+        <v>208</v>
+      </c>
+      <c r="C15" s="20" t="s">
         <v>209</v>
       </c>
-      <c r="C15" s="20" t="s">
-        <v>210</v>
-      </c>
       <c r="D15" s="20" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E15" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D15,Clubs!$A$2:$A$20,0)),"")</f>
         <v>FUK</v>
       </c>
       <c r="F15" s="20" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G15" s="20" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="H15" s="20"/>
       <c r="I15" s="20"/>
@@ -4568,23 +4514,23 @@
         <v>Guillaume PASQUET</v>
       </c>
       <c r="B16" s="20" t="s">
+        <v>210</v>
+      </c>
+      <c r="C16" s="20" t="s">
         <v>211</v>
       </c>
-      <c r="C16" s="20" t="s">
-        <v>212</v>
-      </c>
       <c r="D16" s="20" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E16" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D16,Clubs!$A$2:$A$20,0)),"")</f>
         <v>FUK</v>
       </c>
       <c r="F16" s="20" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G16" s="20" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="H16" s="20"/>
       <c r="I16" s="20"/>
@@ -4597,7 +4543,7 @@
         <v>0</v>
       </c>
       <c r="M16" s="20" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4606,23 +4552,23 @@
         <v>Inès ICHARD</v>
       </c>
       <c r="B17" s="20" t="s">
+        <v>212</v>
+      </c>
+      <c r="C17" s="20" t="s">
         <v>213</v>
       </c>
-      <c r="C17" s="20" t="s">
-        <v>214</v>
-      </c>
       <c r="D17" s="20" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E17" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D17,Clubs!$A$2:$A$20,0)),"")</f>
         <v>FUK</v>
       </c>
       <c r="F17" s="20" t="s">
+        <v>182</v>
+      </c>
+      <c r="G17" s="20" t="s">
         <v>183</v>
-      </c>
-      <c r="G17" s="20" t="s">
-        <v>184</v>
       </c>
       <c r="H17" s="20"/>
       <c r="I17" s="20"/>
@@ -4642,20 +4588,20 @@
         <v>Iris VENDOMÈLE</v>
       </c>
       <c r="B18" s="20" t="s">
+        <v>214</v>
+      </c>
+      <c r="C18" s="20" t="s">
         <v>215</v>
       </c>
-      <c r="C18" s="20" t="s">
-        <v>216</v>
-      </c>
       <c r="D18" s="20" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E18" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D18,Clubs!$A$2:$A$20,0)),"")</f>
         <v>FUK</v>
       </c>
       <c r="F18" s="20" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G18" s="20" t="s">
         <v>25</v>
@@ -4678,23 +4624,23 @@
         <v>Kiria BOYER</v>
       </c>
       <c r="B19" s="20" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C19" s="20" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="D19" s="20" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E19" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D19,Clubs!$A$2:$A$20,0)),"")</f>
         <v>FUK</v>
       </c>
       <c r="F19" s="20" t="s">
+        <v>182</v>
+      </c>
+      <c r="G19" s="20" t="s">
         <v>183</v>
-      </c>
-      <c r="G19" s="20" t="s">
-        <v>184</v>
       </c>
       <c r="H19" s="20"/>
       <c r="I19" s="20"/>
@@ -4714,20 +4660,20 @@
         <v>Liam PROST</v>
       </c>
       <c r="B20" s="20" t="s">
+        <v>217</v>
+      </c>
+      <c r="C20" s="20" t="s">
         <v>218</v>
       </c>
-      <c r="C20" s="20" t="s">
-        <v>219</v>
-      </c>
       <c r="D20" s="20" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E20" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D20,Clubs!$A$2:$A$20,0)),"")</f>
         <v>FUK</v>
       </c>
       <c r="F20" s="20" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G20" s="20" t="s">
         <v>46</v>
@@ -4750,20 +4696,20 @@
         <v>Logan PROST</v>
       </c>
       <c r="B21" s="20" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C21" s="20" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D21" s="20" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E21" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D21,Clubs!$A$2:$A$20,0)),"")</f>
         <v>FUK</v>
       </c>
       <c r="F21" s="20" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G21" s="20" t="s">
         <v>25</v>
@@ -4786,20 +4732,20 @@
         <v>Mahé PASQUET</v>
       </c>
       <c r="B22" s="20" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C22" s="20" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D22" s="20" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E22" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D22,Clubs!$A$2:$A$20,0)),"")</f>
         <v>FUK</v>
       </c>
       <c r="F22" s="20" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G22" s="20" t="s">
         <v>46</v>
@@ -4825,17 +4771,17 @@
         <v>66</v>
       </c>
       <c r="C23" s="20" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="D23" s="20" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E23" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D23,Clubs!$A$2:$A$20,0)),"")</f>
         <v>FUK</v>
       </c>
       <c r="F23" s="20" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G23" s="20" t="s">
         <v>46</v>
@@ -4858,23 +4804,23 @@
         <v>Pierre RODRIGUE</v>
       </c>
       <c r="B24" s="20" t="s">
+        <v>222</v>
+      </c>
+      <c r="C24" s="20" t="s">
         <v>223</v>
       </c>
-      <c r="C24" s="20" t="s">
-        <v>224</v>
-      </c>
       <c r="D24" s="20" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E24" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D24,Clubs!$A$2:$A$20,0)),"")</f>
         <v>FUK</v>
       </c>
       <c r="F24" s="20" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G24" s="20" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="H24" s="20"/>
       <c r="I24" s="20"/>
@@ -4894,23 +4840,23 @@
         <v>Salim YOUSSOUF</v>
       </c>
       <c r="B25" s="20" t="s">
+        <v>224</v>
+      </c>
+      <c r="C25" s="20" t="s">
         <v>225</v>
       </c>
-      <c r="C25" s="20" t="s">
-        <v>226</v>
-      </c>
       <c r="D25" s="20" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E25" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D25,Clubs!$A$2:$A$20,0)),"")</f>
         <v>FUK</v>
       </c>
       <c r="F25" s="20" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G25" s="20" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="H25" s="20"/>
       <c r="I25" s="20"/>
@@ -4923,7 +4869,7 @@
         <v>0</v>
       </c>
       <c r="M25" s="20" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4932,23 +4878,23 @@
         <v>Sébastien ELIE</v>
       </c>
       <c r="B26" s="20" t="s">
+        <v>226</v>
+      </c>
+      <c r="C26" s="20" t="s">
         <v>227</v>
       </c>
-      <c r="C26" s="20" t="s">
-        <v>228</v>
-      </c>
       <c r="D26" s="20" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E26" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D26,Clubs!$A$2:$A$20,0)),"")</f>
         <v>FUK</v>
       </c>
       <c r="F26" s="20" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G26" s="20" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="H26" s="20"/>
       <c r="I26" s="20"/>
@@ -4961,7 +4907,7 @@
         <v>0</v>
       </c>
       <c r="M26" s="20" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4970,24 +4916,24 @@
         <v>Alexandre</v>
       </c>
       <c r="B27" s="20" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C27" s="20"/>
       <c r="D27" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E27" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D27,Clubs!$A$2:$A$20,0)),"")</f>
         <v>MAN</v>
       </c>
       <c r="F27" s="20" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G27" s="20" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="H27" s="20" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="I27" s="20" t="n">
         <v>100</v>
@@ -5001,7 +4947,7 @@
         <v>0</v>
       </c>
       <c r="M27" s="20" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5010,24 +4956,24 @@
         <v>Cédric</v>
       </c>
       <c r="B28" s="20" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="C28" s="20"/>
       <c r="D28" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E28" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D28,Clubs!$A$2:$A$20,0)),"")</f>
         <v>MAN</v>
       </c>
       <c r="F28" s="20" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G28" s="20" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="H28" s="20" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="I28" s="20" t="n">
         <v>91.8</v>
@@ -5052,14 +4998,14 @@
       </c>
       <c r="C29" s="20"/>
       <c r="D29" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E29" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D29,Clubs!$A$2:$A$20,0)),"")</f>
         <v>MAN</v>
       </c>
       <c r="F29" s="20" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G29" s="20" t="s">
         <v>46</v>
@@ -5082,23 +5028,23 @@
         <v>Eve RIVIERE</v>
       </c>
       <c r="B30" s="20" t="s">
+        <v>233</v>
+      </c>
+      <c r="C30" s="20" t="s">
         <v>234</v>
       </c>
-      <c r="C30" s="20" t="s">
-        <v>235</v>
-      </c>
       <c r="D30" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E30" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D30,Clubs!$A$2:$A$20,0)),"")</f>
         <v>MAN</v>
       </c>
       <c r="F30" s="20" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G30" s="20" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="H30" s="20"/>
       <c r="I30" s="20" t="n">
@@ -5124,17 +5070,17 @@
       </c>
       <c r="C31" s="20"/>
       <c r="D31" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E31" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D31,Clubs!$A$2:$A$20,0)),"")</f>
         <v>MAN</v>
       </c>
       <c r="F31" s="20" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G31" s="20" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="H31" s="20"/>
       <c r="I31" s="20"/>
@@ -5154,20 +5100,20 @@
         <v>Lily BEGUE</v>
       </c>
       <c r="B32" s="20" t="s">
+        <v>235</v>
+      </c>
+      <c r="C32" s="20" t="s">
         <v>236</v>
       </c>
-      <c r="C32" s="20" t="s">
-        <v>237</v>
-      </c>
       <c r="D32" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E32" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D32,Clubs!$A$2:$A$20,0)),"")</f>
         <v>MAN</v>
       </c>
       <c r="F32" s="20" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G32" s="20" t="s">
         <v>46</v>
@@ -5192,20 +5138,20 @@
         <v>Lucie PAYET</v>
       </c>
       <c r="B33" s="20" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C33" s="20" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D33" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E33" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D33,Clubs!$A$2:$A$20,0)),"")</f>
         <v>MAN</v>
       </c>
       <c r="F33" s="20" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G33" s="20" t="s">
         <v>46</v>
@@ -5230,24 +5176,24 @@
         <v>Mathias</v>
       </c>
       <c r="B34" s="20" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C34" s="20"/>
       <c r="D34" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E34" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D34,Clubs!$A$2:$A$20,0)),"")</f>
         <v>MAN</v>
       </c>
       <c r="F34" s="20" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G34" s="20" t="s">
+        <v>186</v>
+      </c>
+      <c r="H34" s="20" t="s">
         <v>187</v>
-      </c>
-      <c r="H34" s="20" t="s">
-        <v>188</v>
       </c>
       <c r="I34" s="20" t="n">
         <v>76.2</v>
@@ -5272,17 +5218,17 @@
       </c>
       <c r="C35" s="20"/>
       <c r="D35" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E35" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D35,Clubs!$A$2:$A$20,0)),"")</f>
         <v>MAN</v>
       </c>
       <c r="F35" s="20" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G35" s="20" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="H35" s="20"/>
       <c r="I35" s="20"/>
@@ -5302,24 +5248,24 @@
         <v>Théo</v>
       </c>
       <c r="B36" s="20" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C36" s="20"/>
       <c r="D36" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E36" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D36,Clubs!$A$2:$A$20,0)),"")</f>
         <v>MAN</v>
       </c>
       <c r="F36" s="20" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G36" s="20" t="s">
+        <v>186</v>
+      </c>
+      <c r="H36" s="20" t="s">
         <v>187</v>
-      </c>
-      <c r="H36" s="20" t="s">
-        <v>188</v>
       </c>
       <c r="I36" s="20" t="n">
         <v>60.5</v>
@@ -5344,17 +5290,17 @@
       </c>
       <c r="C37" s="20"/>
       <c r="D37" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E37" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D37,Clubs!$A$2:$A$20,0)),"")</f>
         <v>MAN</v>
       </c>
       <c r="F37" s="20" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G37" s="20" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="H37" s="20"/>
       <c r="I37" s="20"/>
@@ -5374,23 +5320,23 @@
         <v>Ambre BEAUVOIR</v>
       </c>
       <c r="B38" s="20" t="s">
+        <v>240</v>
+      </c>
+      <c r="C38" s="20" t="s">
         <v>241</v>
       </c>
-      <c r="C38" s="20" t="s">
+      <c r="D38" s="20" t="s">
         <v>242</v>
-      </c>
-      <c r="D38" s="20" t="s">
-        <v>243</v>
       </c>
       <c r="E38" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D38,Clubs!$A$2:$A$20,0)),"")</f>
         <v>SHO</v>
       </c>
       <c r="F38" s="20" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G38" s="20" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="H38" s="20"/>
       <c r="I38" s="20"/>
@@ -5410,34 +5356,34 @@
         <v>Chloé FONTAINE</v>
       </c>
       <c r="B39" s="20" t="s">
+        <v>243</v>
+      </c>
+      <c r="C39" s="20" t="s">
         <v>244</v>
       </c>
-      <c r="C39" s="20" t="s">
-        <v>245</v>
-      </c>
       <c r="D39" s="20" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E39" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D39,Clubs!$A$2:$A$20,0)),"")</f>
         <v>SHO</v>
       </c>
       <c r="F39" s="20" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G39" s="20"/>
       <c r="H39" s="20"/>
       <c r="I39" s="20"/>
       <c r="J39" s="20"/>
       <c r="K39" s="20" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="L39" s="22" t="n">
         <f aca="false">COUNTIF('Fight card'!$I$6:$I$200,A39)+COUNTIF('Fight card'!$K$6:$K$200,A39)</f>
         <v>1</v>
       </c>
       <c r="M39" s="20" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5446,23 +5392,23 @@
         <v>Emmanuelle GRUCHET</v>
       </c>
       <c r="B40" s="20" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C40" s="20" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D40" s="20" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E40" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D40,Clubs!$A$2:$A$20,0)),"")</f>
         <v>SHO</v>
       </c>
       <c r="F40" s="20" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G40" s="20" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="H40" s="20"/>
       <c r="I40" s="20"/>
@@ -5482,26 +5428,26 @@
         <v>Ethan BÉGUÉ</v>
       </c>
       <c r="B41" s="20" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C41" s="20" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="D41" s="20" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E41" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D41,Clubs!$A$2:$A$20,0)),"")</f>
         <v>SHO</v>
       </c>
       <c r="F41" s="20" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G41" s="20" t="s">
         <v>46</v>
       </c>
       <c r="H41" s="20" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I41" s="20"/>
       <c r="J41" s="20"/>
@@ -5520,29 +5466,29 @@
         <v>Jean-Marc SERGE</v>
       </c>
       <c r="B42" s="20" t="s">
+        <v>249</v>
+      </c>
+      <c r="C42" s="20" t="s">
         <v>250</v>
       </c>
-      <c r="C42" s="20" t="s">
-        <v>251</v>
-      </c>
       <c r="D42" s="20" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E42" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D42,Clubs!$A$2:$A$20,0)),"")</f>
         <v>SHO</v>
       </c>
       <c r="F42" s="20" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G42" s="20" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="H42" s="20"/>
       <c r="I42" s="20"/>
       <c r="J42" s="20"/>
       <c r="K42" s="20" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="L42" s="22" t="n">
         <f aca="false">COUNTIF('Fight card'!$I$6:$I$200,A42)+COUNTIF('Fight card'!$K$6:$K$200,A42)</f>
@@ -5556,23 +5502,23 @@
         <v>Lanah BARDINOT</v>
       </c>
       <c r="B43" s="20" t="s">
+        <v>251</v>
+      </c>
+      <c r="C43" s="20" t="s">
         <v>252</v>
       </c>
-      <c r="C43" s="20" t="s">
-        <v>253</v>
-      </c>
       <c r="D43" s="20" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E43" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D43,Clubs!$A$2:$A$20,0)),"")</f>
         <v>SHO</v>
       </c>
       <c r="F43" s="20" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G43" s="20" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="H43" s="20"/>
       <c r="I43" s="20"/>
@@ -5592,29 +5538,29 @@
         <v>Mathéo GABRIEL</v>
       </c>
       <c r="B44" s="20" t="s">
+        <v>253</v>
+      </c>
+      <c r="C44" s="20" t="s">
         <v>254</v>
       </c>
-      <c r="C44" s="20" t="s">
-        <v>255</v>
-      </c>
       <c r="D44" s="20" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E44" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D44,Clubs!$A$2:$A$20,0)),"")</f>
         <v>SHO</v>
       </c>
       <c r="F44" s="20" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G44" s="20" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="H44" s="20"/>
       <c r="I44" s="20"/>
       <c r="J44" s="20"/>
       <c r="K44" s="20" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="L44" s="22" t="n">
         <f aca="false">COUNTIF('Fight card'!$I$6:$I$200,A44)+COUNTIF('Fight card'!$K$6:$K$200,A44)</f>
@@ -5628,29 +5574,29 @@
         <v>Miguel IBAO</v>
       </c>
       <c r="B45" s="20" t="s">
+        <v>255</v>
+      </c>
+      <c r="C45" s="20" t="s">
         <v>256</v>
       </c>
-      <c r="C45" s="20" t="s">
-        <v>257</v>
-      </c>
       <c r="D45" s="20" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E45" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D45,Clubs!$A$2:$A$20,0)),"")</f>
         <v>SHO</v>
       </c>
       <c r="F45" s="20" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G45" s="20" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="H45" s="20"/>
       <c r="I45" s="20"/>
       <c r="J45" s="20"/>
       <c r="K45" s="20" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="L45" s="22" t="n">
         <f aca="false">COUNTIF('Fight card'!$I$6:$I$200,A45)+COUNTIF('Fight card'!$K$6:$K$200,A45)</f>
@@ -5664,26 +5610,26 @@
         <v>Thomas GUICHARD</v>
       </c>
       <c r="B46" s="20" t="s">
+        <v>257</v>
+      </c>
+      <c r="C46" s="20" t="s">
         <v>258</v>
       </c>
-      <c r="C46" s="20" t="s">
-        <v>259</v>
-      </c>
       <c r="D46" s="20" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E46" s="21" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D46,Clubs!$A$2:$A$20,0)),"")</f>
         <v>SHO</v>
       </c>
       <c r="F46" s="20" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G46" s="20" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="H46" s="20" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="I46" s="20" t="n">
         <v>84</v>
@@ -5734,39 +5680,39 @@
         <v>15</v>
       </c>
       <c r="B1" s="19" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="20" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B2" s="20" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B3" s="20" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="20" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="20" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fight card recalibrée au poids : 3 kg max enfants, 5 kg max adultes (26 combats)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BG94EkAj2aYi3kCmvbMWy9
</commit_message>
<xml_diff>
--- a/dojo/interclub/shidokan-challenge-974-fight-card.xlsx
+++ b/dojo/interclub/shidokan-challenge-974-fight-card.xlsx
@@ -14,9 +14,9 @@
     <sheet name="Clubs" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Combattants!$A$1:$M$51</definedName>
+    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Combattants!$A$1:$M$52</definedName>
     <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Titles" vbProcedure="false">'Fight card'!$5:$5</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Fight card'!$A$5:$R$33</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Fight card'!$A$5:$R$31</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="630" uniqueCount="282">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="617" uniqueCount="278">
   <si>
     <t xml:space="preserve">SHIDOKAN CHALLENGE 974 — ORDRE DES COMBATS</t>
   </si>
@@ -382,28 +382,40 @@
     <t xml:space="preserve">THEO FONTAINE</t>
   </si>
   <si>
-    <t xml:space="preserve">Seniors H 78-84 kg</t>
+    <t xml:space="preserve">Seniors H 78-79 kg</t>
   </si>
   <si>
     <t xml:space="preserve">Sébastien ELIE</t>
   </si>
   <si>
+    <t xml:space="preserve">Guillaume PASQUET</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13h25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MMA -80 kg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Miguel IBAO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MATHIAS DIJOUX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Co-vedette</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seniors H 83-84 kg</t>
+  </si>
+  <si>
     <t xml:space="preserve">Thomas GUICHARD</t>
   </si>
   <si>
-    <t xml:space="preserve">13h25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MMA -80 kg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Miguel IBAO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MATHIAS DIJOUX</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Co-vedette</t>
+    <t xml:space="preserve">Guillaume PAYET</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13h30</t>
   </si>
   <si>
     <t xml:space="preserve">Seniors H 98-100 kg</t>
@@ -415,30 +427,6 @@
     <t xml:space="preserve">CEDRIC PAYET</t>
   </si>
   <si>
-    <t xml:space="preserve">13h30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Seniors H 60-66 kg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jonathan BOYER</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Seniors H 79-84 kg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Guillaume PASQUET</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13h35</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Seniors H 100-106 kg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Salim YOUSSOUF</t>
-  </si>
-  <si>
     <t xml:space="preserve">Combat vedette</t>
   </si>
   <si>
@@ -565,130 +553,130 @@
     <t xml:space="preserve">Cadets</t>
   </si>
   <si>
+    <t xml:space="preserve">Guillaume</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PAYET</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZAMBERNARDI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lorentz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Benjamins</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Melina</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FOLIO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pupilles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exhibition. Catégorie à préciser.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mike</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MIKE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seniors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-80 kg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Raphaël</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FRAYNAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AXEL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DUHOU</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fukkatsu Kyokushin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Basile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ABEL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Benjamin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LEGRAND</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bilal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SALIMA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Minimes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Camilya</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BACAR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Poussins</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clément</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DELMAS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Réparti en -80 kg ou +80 kg à la pesée.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EDEN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BOYER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Elie-Rose</t>
+  </si>
+  <si>
+    <t xml:space="preserve">THOMAS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PASQUET</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inès</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ICHARD</t>
+  </si>
+  <si>
     <t xml:space="preserve">Jonathan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BOYER</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ZAMBERNARDI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lorentz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PAYET</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Benjamins</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Melina</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FOLIO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pupilles</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Exhibition. Catégorie à préciser.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mike</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MIKE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Seniors</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-80 kg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NOA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Raphaël</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FRAYNAL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AXEL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DUHOU</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fukkatsu Kyokushin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Basile</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ABEL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Benjamin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LEGRAND</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bilal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SALIMA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Minimes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Camilya</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BACAR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Poussins</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clément</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DELMAS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Réparti en -80 kg ou +80 kg à la pesée.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EDEN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Elie-Rose</t>
-  </si>
-  <si>
-    <t xml:space="preserve">THOMAS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Guillaume</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PASQUET</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Inès</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ICHARD</t>
   </si>
   <si>
     <t xml:space="preserve">Kiria</t>
@@ -1614,7 +1602,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:R33"/>
+  <dimension ref="A1:R31"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -1646,7 +1634,7 @@
       </c>
       <c r="O1" s="3" t="n">
         <f aca="false">COUNTA(I6:I200)</f>
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1670,7 +1658,7 @@
       </c>
       <c r="O3" s="3" t="n">
         <f aca="false">O1-O2</f>
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2888,7 +2876,7 @@
       </c>
       <c r="L28" s="13" t="str">
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(K28,Combattants!$A$2:$A$200,0)),"")</f>
-        <v>SHO</v>
+        <v>FUK</v>
       </c>
       <c r="M28" s="9" t="s">
         <v>31</v>
@@ -2985,14 +2973,14 @@
       </c>
       <c r="J30" s="13" t="str">
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(I30,Combattants!$A$2:$A$200,0)),"")</f>
-        <v>FUK</v>
+        <v>SHO</v>
       </c>
       <c r="K30" s="14" t="s">
         <v>116</v>
       </c>
       <c r="L30" s="13" t="str">
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(K30,Combattants!$A$2:$A$200,0)),"")</f>
-        <v>MAN</v>
+        <v>FAK</v>
       </c>
       <c r="M30" s="9" t="s">
         <v>31</v>
@@ -3032,18 +3020,18 @@
         <v>95</v>
       </c>
       <c r="I31" s="12" t="s">
-        <v>105</v>
+        <v>119</v>
       </c>
       <c r="J31" s="13" t="str">
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(I31,Combattants!$A$2:$A$200,0)),"")</f>
-        <v>MAN</v>
+        <v>FUK</v>
       </c>
       <c r="K31" s="14" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="L31" s="13" t="str">
         <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(K31,Combattants!$A$2:$A$200,0)),"")</f>
-        <v>FAK</v>
+        <v>MAN</v>
       </c>
       <c r="M31" s="9" t="s">
         <v>31</v>
@@ -3055,114 +3043,12 @@
       </c>
       <c r="P31" s="9"/>
       <c r="Q31" s="9"/>
-      <c r="R31" s="11"/>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="9" t="n">
-        <v>27</v>
-      </c>
-      <c r="B32" s="9" t="s">
-        <v>117</v>
-      </c>
-      <c r="C32" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="D32" s="10" t="s">
-        <v>93</v>
-      </c>
-      <c r="E32" s="11" t="s">
-        <v>120</v>
-      </c>
-      <c r="F32" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="G32" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="H32" s="10" t="s">
-        <v>95</v>
-      </c>
-      <c r="I32" s="12" t="s">
+      <c r="R31" s="11" t="s">
         <v>121</v>
       </c>
-      <c r="J32" s="13" t="str">
-        <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(I32,Combattants!$A$2:$A$200,0)),"")</f>
-        <v>FUK</v>
-      </c>
-      <c r="K32" s="14" t="s">
-        <v>108</v>
-      </c>
-      <c r="L32" s="13" t="str">
-        <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(K32,Combattants!$A$2:$A$200,0)),"")</f>
-        <v>SHO</v>
-      </c>
-      <c r="M32" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="N32" s="9"/>
-      <c r="O32" s="13" t="str">
-        <f aca="false">IF(N32="Rouge",I32,IF(N32="Bleu",K32,IF(N32="Nul","Match nul","")))</f>
-        <v/>
-      </c>
-      <c r="P32" s="9"/>
-      <c r="Q32" s="9"/>
-      <c r="R32" s="11"/>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="9" t="n">
-        <v>28</v>
-      </c>
-      <c r="B33" s="9" t="s">
-        <v>122</v>
-      </c>
-      <c r="C33" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="D33" s="10" t="s">
-        <v>93</v>
-      </c>
-      <c r="E33" s="11" t="s">
-        <v>123</v>
-      </c>
-      <c r="F33" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="G33" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="H33" s="10" t="s">
-        <v>95</v>
-      </c>
-      <c r="I33" s="12" t="s">
-        <v>116</v>
-      </c>
-      <c r="J33" s="13" t="str">
-        <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(I33,Combattants!$A$2:$A$200,0)),"")</f>
-        <v>MAN</v>
-      </c>
-      <c r="K33" s="14" t="s">
-        <v>124</v>
-      </c>
-      <c r="L33" s="13" t="str">
-        <f aca="false">IFERROR(INDEX(Combattants!$E$2:$E$200,MATCH(K33,Combattants!$A$2:$A$200,0)),"")</f>
-        <v>FUK</v>
-      </c>
-      <c r="M33" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="N33" s="9"/>
-      <c r="O33" s="13" t="str">
-        <f aca="false">IF(N33="Rouge",I33,IF(N33="Bleu",K33,IF(N33="Nul","Match nul","")))</f>
-        <v/>
-      </c>
-      <c r="P33" s="9"/>
-      <c r="Q33" s="9"/>
-      <c r="R33" s="11" t="s">
-        <v>125</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:R33"/>
+  <autoFilter ref="A5:R31"/>
   <conditionalFormatting sqref="A6:R200">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
       <formula>$M6="Terminé"</formula>
@@ -3238,47 +3124,47 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="16" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="B1" s="17" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="16" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="16" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="16" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="B6" s="17" t="n">
         <v>2</v>
@@ -3286,10 +3172,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3297,39 +3183,39 @@
         <v>7</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="19" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="19" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="B11" s="19" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="19" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="B12" s="19" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="19" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="B13" s="19" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3337,20 +3223,20 @@
         <v>92</v>
       </c>
       <c r="B14" s="19" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="19" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="B15" s="19" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
     </row>
   </sheetData>
@@ -3369,7 +3255,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M51"/>
+  <dimension ref="A1:M52"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
@@ -3387,40 +3273,40 @@
   <sheetData>
     <row r="1" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="D1" s="6" t="s">
         <v>15</v>
       </c>
       <c r="E1" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="I1" s="6" t="s">
         <v>155</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="J1" s="6" t="s">
         <v>156</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="K1" s="6" t="s">
         <v>157</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="L1" s="6" t="s">
         <v>158</v>
-      </c>
-      <c r="I1" s="6" t="s">
-        <v>159</v>
-      </c>
-      <c r="J1" s="6" t="s">
-        <v>160</v>
-      </c>
-      <c r="K1" s="6" t="s">
-        <v>161</v>
-      </c>
-      <c r="L1" s="6" t="s">
-        <v>162</v>
       </c>
       <c r="M1" s="6" t="s">
         <v>22</v>
@@ -3432,26 +3318,28 @@
         <v>Ethan ICAZE</v>
       </c>
       <c r="B2" s="19" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="C2" s="19" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="D2" s="19" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="E2" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D2,Clubs!$A$2:$A$20,0)),"")</f>
         <v>FAK</v>
       </c>
       <c r="F2" s="19" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="G2" s="19" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
+      <c r="I2" s="19" t="n">
+        <v>74</v>
+      </c>
       <c r="J2" s="19"/>
       <c r="K2" s="19" t="s">
         <v>27</v>
@@ -3465,32 +3353,32 @@
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="20" t="str">
         <f aca="false">TRIM(B3&amp;" "&amp;C3)</f>
-        <v>Jonathan BOYER</v>
+        <v>Guillaume PAYET</v>
       </c>
       <c r="B3" s="19" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="C3" s="19" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="D3" s="19" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="E3" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D3,Clubs!$A$2:$A$20,0)),"")</f>
         <v>FAK</v>
       </c>
       <c r="F3" s="19" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="G3" s="19"/>
       <c r="H3" s="19"/>
       <c r="I3" s="19" t="n">
-        <v>66</v>
+        <v>83</v>
       </c>
       <c r="J3" s="19"/>
       <c r="K3" s="19" t="s">
-        <v>27</v>
+        <v>99</v>
       </c>
       <c r="L3" s="21" t="n">
         <f aca="false">COUNTIF('Fight card'!$I$6:$I$200,A3)+COUNTIF('Fight card'!$K$6:$K$200,A3)</f>
@@ -3504,20 +3392,20 @@
         <v>Keo ZAMBERNARDI</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="D4" s="19" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="E4" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D4,Clubs!$A$2:$A$20,0)),"")</f>
         <v>FAK</v>
       </c>
       <c r="F4" s="19" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="G4" s="19"/>
       <c r="H4" s="19"/>
@@ -3540,23 +3428,23 @@
         <v>Lorentz PAYET</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="C5" s="19" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="D5" s="19" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="E5" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D5,Clubs!$A$2:$A$20,0)),"")</f>
         <v>FAK</v>
       </c>
       <c r="F5" s="19" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="G5" s="19" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="H5" s="19"/>
       <c r="I5" s="19" t="n">
@@ -3578,23 +3466,23 @@
         <v>Melina FOLIO</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="D6" s="19" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="E6" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D6,Clubs!$A$2:$A$20,0)),"")</f>
         <v>FAK</v>
       </c>
       <c r="F6" s="19" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="G6" s="19" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="H6" s="19"/>
       <c r="I6" s="19" t="n">
@@ -3609,7 +3497,7 @@
         <v>1</v>
       </c>
       <c r="M6" s="19" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3618,26 +3506,26 @@
         <v>Mike MIKE</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="D7" s="19" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="E7" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D7,Clubs!$A$2:$A$20,0)),"")</f>
         <v>FAK</v>
       </c>
       <c r="F7" s="19" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="G7" s="19" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="H7" s="19" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="I7" s="19" t="n">
         <v>59</v>
@@ -3658,20 +3546,20 @@
         <v>NOA ZAMBERNARDI</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="D8" s="19" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="E8" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D8,Clubs!$A$2:$A$20,0)),"")</f>
         <v>FAK</v>
       </c>
       <c r="F8" s="19" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="G8" s="19"/>
       <c r="H8" s="19"/>
@@ -3694,23 +3582,23 @@
         <v>Raphaël FRAYNAL</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="D9" s="19" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="E9" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D9,Clubs!$A$2:$A$20,0)),"")</f>
         <v>FAK</v>
       </c>
       <c r="F9" s="19" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="G9" s="19" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="H9" s="19"/>
       <c r="I9" s="19" t="n">
@@ -3732,20 +3620,20 @@
         <v>AXEL DUHOU</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="D10" s="19" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="E10" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D10,Clubs!$A$2:$A$20,0)),"")</f>
         <v>FUK</v>
       </c>
       <c r="F10" s="19" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="G10" s="19"/>
       <c r="H10" s="19"/>
@@ -3768,23 +3656,23 @@
         <v>Basile ABEL</v>
       </c>
       <c r="B11" s="19" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="D11" s="19" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="E11" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D11,Clubs!$A$2:$A$20,0)),"")</f>
         <v>FUK</v>
       </c>
       <c r="F11" s="19" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="G11" s="19" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="H11" s="19"/>
       <c r="I11" s="19" t="n">
@@ -3806,23 +3694,23 @@
         <v>Benjamin LEGRAND</v>
       </c>
       <c r="B12" s="19" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="D12" s="19" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="E12" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D12,Clubs!$A$2:$A$20,0)),"")</f>
         <v>FUK</v>
       </c>
       <c r="F12" s="19" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="G12" s="19" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="H12" s="19"/>
       <c r="I12" s="19" t="n">
@@ -3844,23 +3732,23 @@
         <v>Bilal SALIMA</v>
       </c>
       <c r="B13" s="19" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="C13" s="19" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="D13" s="19" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="E13" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D13,Clubs!$A$2:$A$20,0)),"")</f>
         <v>FUK</v>
       </c>
       <c r="F13" s="19" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="G13" s="19" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="H13" s="19"/>
       <c r="I13" s="19" t="n">
@@ -3882,23 +3770,23 @@
         <v>Camilya BACAR</v>
       </c>
       <c r="B14" s="19" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="D14" s="19" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="E14" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D14,Clubs!$A$2:$A$20,0)),"")</f>
         <v>FUK</v>
       </c>
       <c r="F14" s="19" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="G14" s="19" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="H14" s="19"/>
       <c r="I14" s="19" t="n">
@@ -3920,23 +3808,23 @@
         <v>Clément DELMAS</v>
       </c>
       <c r="B15" s="19" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="C15" s="19" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="D15" s="19" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="E15" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D15,Clubs!$A$2:$A$20,0)),"")</f>
         <v>FUK</v>
       </c>
       <c r="F15" s="19" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="G15" s="19" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="H15" s="19"/>
       <c r="I15" s="19" t="n">
@@ -3951,7 +3839,7 @@
         <v>1</v>
       </c>
       <c r="M15" s="19" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3960,20 +3848,20 @@
         <v>EDEN BOYER</v>
       </c>
       <c r="B16" s="19" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="C16" s="19" t="s">
-        <v>168</v>
+        <v>198</v>
       </c>
       <c r="D16" s="19" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="E16" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D16,Clubs!$A$2:$A$20,0)),"")</f>
         <v>FUK</v>
       </c>
       <c r="F16" s="19" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="G16" s="19"/>
       <c r="H16" s="19"/>
@@ -3996,23 +3884,23 @@
         <v>Elie-Rose THOMAS</v>
       </c>
       <c r="B17" s="19" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="C17" s="19" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="D17" s="19" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="E17" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D17,Clubs!$A$2:$A$20,0)),"")</f>
         <v>FUK</v>
       </c>
       <c r="F17" s="19" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="G17" s="19" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="H17" s="19"/>
       <c r="I17" s="19" t="n">
@@ -4034,23 +3922,23 @@
         <v>Guillaume PASQUET</v>
       </c>
       <c r="B18" s="19" t="s">
-        <v>205</v>
+        <v>163</v>
       </c>
       <c r="C18" s="19" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="D18" s="19" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="E18" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D18,Clubs!$A$2:$A$20,0)),"")</f>
         <v>FUK</v>
       </c>
       <c r="F18" s="19" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="G18" s="19" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="H18" s="19"/>
       <c r="I18" s="19" t="n">
@@ -4065,7 +3953,7 @@
         <v>1</v>
       </c>
       <c r="M18" s="19" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4074,23 +3962,23 @@
         <v>Inès ICHARD</v>
       </c>
       <c r="B19" s="19" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="C19" s="19" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="D19" s="19" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="E19" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D19,Clubs!$A$2:$A$20,0)),"")</f>
         <v>FUK</v>
       </c>
       <c r="F19" s="19" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="G19" s="19" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="H19" s="19"/>
       <c r="I19" s="19" t="n">
@@ -4109,30 +3997,28 @@
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="20" t="str">
         <f aca="false">TRIM(B20&amp;" "&amp;C20)</f>
-        <v>Kiria BOYER</v>
+        <v>Jonathan BOYER</v>
       </c>
       <c r="B20" s="19" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="C20" s="19" t="s">
-        <v>168</v>
+        <v>198</v>
       </c>
       <c r="D20" s="19" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="E20" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D20,Clubs!$A$2:$A$20,0)),"")</f>
         <v>FUK</v>
       </c>
       <c r="F20" s="19" t="s">
-        <v>176</v>
-      </c>
-      <c r="G20" s="19" t="s">
-        <v>177</v>
-      </c>
+        <v>161</v>
+      </c>
+      <c r="G20" s="19"/>
       <c r="H20" s="19"/>
       <c r="I20" s="19" t="n">
-        <v>23</v>
+        <v>66</v>
       </c>
       <c r="J20" s="19"/>
       <c r="K20" s="19" t="s">
@@ -4140,37 +4026,37 @@
       </c>
       <c r="L20" s="21" t="n">
         <f aca="false">COUNTIF('Fight card'!$I$6:$I$200,A20)+COUNTIF('Fight card'!$K$6:$K$200,A20)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M20" s="19"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="20" t="str">
         <f aca="false">TRIM(B21&amp;" "&amp;C21)</f>
-        <v>Liam PROST</v>
+        <v>Kiria BOYER</v>
       </c>
       <c r="B21" s="19" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="C21" s="19" t="s">
-        <v>211</v>
+        <v>198</v>
       </c>
       <c r="D21" s="19" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="E21" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D21,Clubs!$A$2:$A$20,0)),"")</f>
         <v>FUK</v>
       </c>
       <c r="F21" s="19" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="G21" s="19" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="H21" s="19"/>
       <c r="I21" s="19" t="n">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="J21" s="19"/>
       <c r="K21" s="19" t="s">
@@ -4185,30 +4071,30 @@
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="20" t="str">
         <f aca="false">TRIM(B22&amp;" "&amp;C22)</f>
-        <v>Logan PROST</v>
+        <v>Liam PROST</v>
       </c>
       <c r="B22" s="19" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="C22" s="19" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="D22" s="19" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="E22" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D22,Clubs!$A$2:$A$20,0)),"")</f>
         <v>FUK</v>
       </c>
       <c r="F22" s="19" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="G22" s="19" t="s">
-        <v>198</v>
+        <v>168</v>
       </c>
       <c r="H22" s="19"/>
       <c r="I22" s="19" t="n">
-        <v>23</v>
+        <v>38</v>
       </c>
       <c r="J22" s="19"/>
       <c r="K22" s="19" t="s">
@@ -4223,30 +4109,30 @@
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="20" t="str">
         <f aca="false">TRIM(B23&amp;" "&amp;C23)</f>
-        <v>Mahé PASQUET</v>
+        <v>Logan PROST</v>
       </c>
       <c r="B23" s="19" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="C23" s="19" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D23" s="19" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="E23" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D23,Clubs!$A$2:$A$20,0)),"")</f>
         <v>FUK</v>
       </c>
       <c r="F23" s="19" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="G23" s="19" t="s">
-        <v>173</v>
+        <v>193</v>
       </c>
       <c r="H23" s="19"/>
       <c r="I23" s="19" t="n">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="J23" s="19"/>
       <c r="K23" s="19" t="s">
@@ -4261,26 +4147,26 @@
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="20" t="str">
         <f aca="false">TRIM(B24&amp;" "&amp;C24)</f>
-        <v>Nathan BABEF</v>
+        <v>Mahé PASQUET</v>
       </c>
       <c r="B24" s="19" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="C24" s="19" t="s">
-        <v>215</v>
+        <v>201</v>
       </c>
       <c r="D24" s="19" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="E24" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D24,Clubs!$A$2:$A$20,0)),"")</f>
         <v>FUK</v>
       </c>
       <c r="F24" s="19" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="G24" s="19" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="H24" s="19"/>
       <c r="I24" s="19" t="n">
@@ -4299,30 +4185,30 @@
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="20" t="str">
         <f aca="false">TRIM(B25&amp;" "&amp;C25)</f>
-        <v>Pierre RODRIGUE</v>
+        <v>Nathan BABEF</v>
       </c>
       <c r="B25" s="19" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="C25" s="19" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="D25" s="19" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="E25" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D25,Clubs!$A$2:$A$20,0)),"")</f>
         <v>FUK</v>
       </c>
       <c r="F25" s="19" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="G25" s="19" t="s">
-        <v>195</v>
+        <v>168</v>
       </c>
       <c r="H25" s="19"/>
       <c r="I25" s="19" t="n">
-        <v>57</v>
+        <v>35</v>
       </c>
       <c r="J25" s="19"/>
       <c r="K25" s="19" t="s">
@@ -4337,30 +4223,30 @@
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="20" t="str">
         <f aca="false">TRIM(B26&amp;" "&amp;C26)</f>
-        <v>Salim YOUSSOUF</v>
+        <v>Pierre RODRIGUE</v>
       </c>
       <c r="B26" s="19" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="C26" s="19" t="s">
-        <v>219</v>
+        <v>213</v>
       </c>
       <c r="D26" s="19" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="E26" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D26,Clubs!$A$2:$A$20,0)),"")</f>
         <v>FUK</v>
       </c>
       <c r="F26" s="19" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="G26" s="19" t="s">
-        <v>181</v>
+        <v>190</v>
       </c>
       <c r="H26" s="19"/>
       <c r="I26" s="19" t="n">
-        <v>106</v>
+        <v>57</v>
       </c>
       <c r="J26" s="19"/>
       <c r="K26" s="19" t="s">
@@ -4370,37 +4256,35 @@
         <f aca="false">COUNTIF('Fight card'!$I$6:$I$200,A26)+COUNTIF('Fight card'!$K$6:$K$200,A26)</f>
         <v>1</v>
       </c>
-      <c r="M26" s="19" t="s">
-        <v>201</v>
-      </c>
+      <c r="M26" s="19"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="20" t="str">
         <f aca="false">TRIM(B27&amp;" "&amp;C27)</f>
-        <v>Sébastien ELIE</v>
+        <v>Salim YOUSSOUF</v>
       </c>
       <c r="B27" s="19" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="C27" s="19" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
       <c r="D27" s="19" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="E27" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D27,Clubs!$A$2:$A$20,0)),"")</f>
         <v>FUK</v>
       </c>
       <c r="F27" s="19" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="G27" s="19" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="H27" s="19"/>
       <c r="I27" s="19" t="n">
-        <v>78</v>
+        <v>106</v>
       </c>
       <c r="J27" s="19"/>
       <c r="K27" s="19" t="s">
@@ -4408,39 +4292,39 @@
       </c>
       <c r="L27" s="21" t="n">
         <f aca="false">COUNTIF('Fight card'!$I$6:$I$200,A27)+COUNTIF('Fight card'!$K$6:$K$200,A27)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M27" s="19" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="20" t="str">
         <f aca="false">TRIM(B28&amp;" "&amp;C28)</f>
-        <v>Antoine RIVIERE</v>
+        <v>Sébastien ELIE</v>
       </c>
       <c r="B28" s="19" t="s">
-        <v>222</v>
+        <v>216</v>
       </c>
       <c r="C28" s="19" t="s">
-        <v>223</v>
+        <v>217</v>
       </c>
       <c r="D28" s="19" t="s">
-        <v>224</v>
+        <v>183</v>
       </c>
       <c r="E28" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D28,Clubs!$A$2:$A$20,0)),"")</f>
-        <v>MAN</v>
+        <v>FUK</v>
       </c>
       <c r="F28" s="19" t="s">
-        <v>165</v>
-      </c>
-      <c r="G28" s="19"/>
-      <c r="H28" s="19" t="s">
-        <v>225</v>
-      </c>
+        <v>161</v>
+      </c>
+      <c r="G28" s="19" t="s">
+        <v>176</v>
+      </c>
+      <c r="H28" s="19"/>
       <c r="I28" s="19" t="n">
-        <v>35</v>
+        <v>78</v>
       </c>
       <c r="J28" s="19"/>
       <c r="K28" s="19" t="s">
@@ -4448,36 +4332,40 @@
       </c>
       <c r="L28" s="21" t="n">
         <f aca="false">COUNTIF('Fight card'!$I$6:$I$200,A28)+COUNTIF('Fight card'!$K$6:$K$200,A28)</f>
-        <v>2</v>
-      </c>
-      <c r="M28" s="19"/>
+        <v>1</v>
+      </c>
+      <c r="M28" s="19" t="s">
+        <v>196</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="20" t="str">
         <f aca="false">TRIM(B29&amp;" "&amp;C29)</f>
-        <v>CEDRIC PAYET</v>
+        <v>Antoine RIVIERE</v>
       </c>
       <c r="B29" s="19" t="s">
-        <v>226</v>
+        <v>218</v>
       </c>
       <c r="C29" s="19" t="s">
-        <v>172</v>
+        <v>219</v>
       </c>
       <c r="D29" s="19" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="E29" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D29,Clubs!$A$2:$A$20,0)),"")</f>
         <v>MAN</v>
       </c>
       <c r="F29" s="19" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="G29" s="19"/>
       <c r="H29" s="19" t="s">
-        <v>227</v>
-      </c>
-      <c r="I29" s="19"/>
+        <v>221</v>
+      </c>
+      <c r="I29" s="19" t="n">
+        <v>35</v>
+      </c>
       <c r="J29" s="19"/>
       <c r="K29" s="19" t="s">
         <v>27</v>
@@ -4491,31 +4379,29 @@
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="20" t="str">
         <f aca="false">TRIM(B30&amp;" "&amp;C30)</f>
-        <v>DOMNOE COUILLAUD</v>
+        <v>CEDRIC PAYET</v>
       </c>
       <c r="B30" s="19" t="s">
-        <v>228</v>
+        <v>222</v>
       </c>
       <c r="C30" s="19" t="s">
-        <v>229</v>
+        <v>164</v>
       </c>
       <c r="D30" s="19" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="E30" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D30,Clubs!$A$2:$A$20,0)),"")</f>
         <v>MAN</v>
       </c>
       <c r="F30" s="19" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="G30" s="19"/>
       <c r="H30" s="19" t="s">
-        <v>230</v>
-      </c>
-      <c r="I30" s="19" t="n">
-        <v>40</v>
-      </c>
+        <v>223</v>
+      </c>
+      <c r="I30" s="19"/>
       <c r="J30" s="19"/>
       <c r="K30" s="19" t="s">
         <v>27</v>
@@ -4529,30 +4415,30 @@
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="20" t="str">
         <f aca="false">TRIM(B31&amp;" "&amp;C31)</f>
-        <v>EVE RIVIERE</v>
+        <v>DOMNOE COUILLAUD</v>
       </c>
       <c r="B31" s="19" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="C31" s="19" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="D31" s="19" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="E31" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D31,Clubs!$A$2:$A$20,0)),"")</f>
         <v>MAN</v>
       </c>
       <c r="F31" s="19" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="G31" s="19"/>
       <c r="H31" s="19" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="I31" s="19" t="n">
-        <v>55</v>
+        <v>40</v>
       </c>
       <c r="J31" s="19"/>
       <c r="K31" s="19" t="s">
@@ -4567,30 +4453,30 @@
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="20" t="str">
         <f aca="false">TRIM(B32&amp;" "&amp;C32)</f>
-        <v>GILLES IDMOND</v>
+        <v>EVE RIVIERE</v>
       </c>
       <c r="B32" s="19" t="s">
-        <v>233</v>
+        <v>227</v>
       </c>
       <c r="C32" s="19" t="s">
-        <v>234</v>
+        <v>219</v>
       </c>
       <c r="D32" s="19" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="E32" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D32,Clubs!$A$2:$A$20,0)),"")</f>
         <v>MAN</v>
       </c>
       <c r="F32" s="19" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="G32" s="19"/>
       <c r="H32" s="19" t="s">
-        <v>235</v>
+        <v>228</v>
       </c>
       <c r="I32" s="19" t="n">
-        <v>74.9</v>
+        <v>55</v>
       </c>
       <c r="J32" s="19"/>
       <c r="K32" s="19" t="s">
@@ -4605,28 +4491,30 @@
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="20" t="str">
         <f aca="false">TRIM(B33&amp;" "&amp;C33)</f>
-        <v>HELENA PAYET</v>
+        <v>GILLES IDMOND</v>
       </c>
       <c r="B33" s="19" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="C33" s="19" t="s">
-        <v>172</v>
+        <v>230</v>
       </c>
       <c r="D33" s="19" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="E33" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D33,Clubs!$A$2:$A$20,0)),"")</f>
         <v>MAN</v>
       </c>
       <c r="F33" s="19" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="G33" s="19"/>
-      <c r="H33" s="19"/>
+      <c r="H33" s="19" t="s">
+        <v>231</v>
+      </c>
       <c r="I33" s="19" t="n">
-        <v>55</v>
+        <v>74.9</v>
       </c>
       <c r="J33" s="19"/>
       <c r="K33" s="19" t="s">
@@ -4641,30 +4529,28 @@
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="20" t="str">
         <f aca="false">TRIM(B34&amp;" "&amp;C34)</f>
-        <v>HUGO GRONDIN</v>
+        <v>HELENA PAYET</v>
       </c>
       <c r="B34" s="19" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="C34" s="19" t="s">
-        <v>238</v>
+        <v>164</v>
       </c>
       <c r="D34" s="19" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="E34" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D34,Clubs!$A$2:$A$20,0)),"")</f>
         <v>MAN</v>
       </c>
       <c r="F34" s="19" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="G34" s="19"/>
-      <c r="H34" s="19" t="s">
-        <v>239</v>
-      </c>
+      <c r="H34" s="19"/>
       <c r="I34" s="19" t="n">
-        <v>35</v>
+        <v>55</v>
       </c>
       <c r="J34" s="19"/>
       <c r="K34" s="19" t="s">
@@ -4679,28 +4565,28 @@
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="20" t="str">
         <f aca="false">TRIM(B35&amp;" "&amp;C35)</f>
-        <v>Lily BEGUE</v>
+        <v>HUGO GRONDIN</v>
       </c>
       <c r="B35" s="19" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="C35" s="19" t="s">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="D35" s="19" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="E35" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D35,Clubs!$A$2:$A$20,0)),"")</f>
         <v>MAN</v>
       </c>
       <c r="F35" s="19" t="s">
-        <v>176</v>
-      </c>
-      <c r="G35" s="19" t="s">
-        <v>173</v>
-      </c>
-      <c r="H35" s="19"/>
+        <v>161</v>
+      </c>
+      <c r="G35" s="19"/>
+      <c r="H35" s="19" t="s">
+        <v>235</v>
+      </c>
       <c r="I35" s="19" t="n">
         <v>35</v>
       </c>
@@ -4710,37 +4596,37 @@
       </c>
       <c r="L35" s="21" t="n">
         <f aca="false">COUNTIF('Fight card'!$I$6:$I$200,A35)+COUNTIF('Fight card'!$K$6:$K$200,A35)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M35" s="19"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="20" t="str">
         <f aca="false">TRIM(B36&amp;" "&amp;C36)</f>
-        <v>Lucie PAYET</v>
+        <v>Lily BEGUE</v>
       </c>
       <c r="B36" s="19" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="C36" s="19" t="s">
-        <v>172</v>
+        <v>237</v>
       </c>
       <c r="D36" s="19" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="E36" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D36,Clubs!$A$2:$A$20,0)),"")</f>
         <v>MAN</v>
       </c>
       <c r="F36" s="19" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="G36" s="19" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="H36" s="19"/>
       <c r="I36" s="19" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="J36" s="19"/>
       <c r="K36" s="19" t="s">
@@ -4748,39 +4634,41 @@
       </c>
       <c r="L36" s="21" t="n">
         <f aca="false">COUNTIF('Fight card'!$I$6:$I$200,A36)+COUNTIF('Fight card'!$K$6:$K$200,A36)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M36" s="19"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="20" t="str">
         <f aca="false">TRIM(B37&amp;" "&amp;C37)</f>
-        <v>MATHIAS DIJOUX</v>
+        <v>Lucie PAYET</v>
       </c>
       <c r="B37" s="19" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="C37" s="19" t="s">
-        <v>244</v>
+        <v>164</v>
       </c>
       <c r="D37" s="19" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="E37" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D37,Clubs!$A$2:$A$20,0)),"")</f>
         <v>MAN</v>
       </c>
       <c r="F37" s="19" t="s">
-        <v>165</v>
-      </c>
-      <c r="G37" s="19"/>
-      <c r="H37" s="19" t="s">
-        <v>245</v>
-      </c>
-      <c r="I37" s="19"/>
+        <v>171</v>
+      </c>
+      <c r="G37" s="19" t="s">
+        <v>168</v>
+      </c>
+      <c r="H37" s="19"/>
+      <c r="I37" s="19" t="n">
+        <v>30</v>
+      </c>
       <c r="J37" s="19"/>
       <c r="K37" s="19" t="s">
-        <v>99</v>
+        <v>27</v>
       </c>
       <c r="L37" s="21" t="n">
         <f aca="false">COUNTIF('Fight card'!$I$6:$I$200,A37)+COUNTIF('Fight card'!$K$6:$K$200,A37)</f>
@@ -4791,68 +4679,64 @@
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="20" t="str">
         <f aca="false">TRIM(B38&amp;" "&amp;C38)</f>
-        <v>Matys LABRUYERE</v>
+        <v>MATHIAS DIJOUX</v>
       </c>
       <c r="B38" s="19" t="s">
-        <v>246</v>
+        <v>239</v>
       </c>
       <c r="C38" s="19" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
       <c r="D38" s="19" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="E38" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D38,Clubs!$A$2:$A$20,0)),"")</f>
         <v>MAN</v>
       </c>
       <c r="F38" s="19" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="G38" s="19"/>
-      <c r="H38" s="19"/>
-      <c r="I38" s="19" t="n">
-        <v>65</v>
-      </c>
+      <c r="H38" s="19" t="s">
+        <v>241</v>
+      </c>
+      <c r="I38" s="19"/>
       <c r="J38" s="19"/>
       <c r="K38" s="19" t="s">
-        <v>27</v>
+        <v>99</v>
       </c>
       <c r="L38" s="21" t="n">
         <f aca="false">COUNTIF('Fight card'!$I$6:$I$200,A38)+COUNTIF('Fight card'!$K$6:$K$200,A38)</f>
         <v>1</v>
       </c>
-      <c r="M38" s="19" t="s">
-        <v>248</v>
-      </c>
+      <c r="M38" s="19"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="20" t="str">
         <f aca="false">TRIM(B39&amp;" "&amp;C39)</f>
-        <v>NATHAN RIVIERE</v>
+        <v>Matys LABRUYERE</v>
       </c>
       <c r="B39" s="19" t="s">
-        <v>249</v>
+        <v>242</v>
       </c>
       <c r="C39" s="19" t="s">
-        <v>223</v>
+        <v>243</v>
       </c>
       <c r="D39" s="19" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="E39" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D39,Clubs!$A$2:$A$20,0)),"")</f>
         <v>MAN</v>
       </c>
       <c r="F39" s="19" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="G39" s="19"/>
-      <c r="H39" s="19" t="s">
-        <v>250</v>
-      </c>
+      <c r="H39" s="19"/>
       <c r="I39" s="19" t="n">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="J39" s="19"/>
       <c r="K39" s="19" t="s">
@@ -4862,35 +4746,37 @@
         <f aca="false">COUNTIF('Fight card'!$I$6:$I$200,A39)+COUNTIF('Fight card'!$K$6:$K$200,A39)</f>
         <v>1</v>
       </c>
-      <c r="M39" s="19"/>
+      <c r="M39" s="19" t="s">
+        <v>244</v>
+      </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="20" t="str">
         <f aca="false">TRIM(B40&amp;" "&amp;C40)</f>
-        <v>ROBIN TURPIN</v>
+        <v>NATHAN RIVIERE</v>
       </c>
       <c r="B40" s="19" t="s">
-        <v>251</v>
+        <v>245</v>
       </c>
       <c r="C40" s="19" t="s">
-        <v>252</v>
+        <v>219</v>
       </c>
       <c r="D40" s="19" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="E40" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D40,Clubs!$A$2:$A$20,0)),"")</f>
         <v>MAN</v>
       </c>
       <c r="F40" s="19" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="G40" s="19"/>
       <c r="H40" s="19" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
       <c r="I40" s="19" t="n">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="J40" s="19"/>
       <c r="K40" s="19" t="s">
@@ -4905,68 +4791,70 @@
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="20" t="str">
         <f aca="false">TRIM(B41&amp;" "&amp;C41)</f>
-        <v>THEO FONTAINE</v>
+        <v>ROBIN TURPIN</v>
       </c>
       <c r="B41" s="19" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
       <c r="C41" s="19" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="D41" s="19" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="E41" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D41,Clubs!$A$2:$A$20,0)),"")</f>
         <v>MAN</v>
       </c>
       <c r="F41" s="19" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="G41" s="19"/>
       <c r="H41" s="19" t="s">
-        <v>256</v>
-      </c>
-      <c r="I41" s="19"/>
+        <v>249</v>
+      </c>
+      <c r="I41" s="19" t="n">
+        <v>60</v>
+      </c>
       <c r="J41" s="19"/>
       <c r="K41" s="19" t="s">
-        <v>257</v>
+        <v>27</v>
       </c>
       <c r="L41" s="21" t="n">
         <f aca="false">COUNTIF('Fight card'!$I$6:$I$200,A41)+COUNTIF('Fight card'!$K$6:$K$200,A41)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M41" s="19"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="20" t="str">
         <f aca="false">TRIM(B42&amp;" "&amp;C42)</f>
-        <v>YVAN BOYER</v>
+        <v>THEO FONTAINE</v>
       </c>
       <c r="B42" s="19" t="s">
-        <v>258</v>
+        <v>250</v>
       </c>
       <c r="C42" s="19" t="s">
-        <v>168</v>
+        <v>251</v>
       </c>
       <c r="D42" s="19" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="E42" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D42,Clubs!$A$2:$A$20,0)),"")</f>
         <v>MAN</v>
       </c>
       <c r="F42" s="19" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="G42" s="19"/>
-      <c r="H42" s="19"/>
-      <c r="I42" s="19" t="n">
-        <v>40</v>
-      </c>
+      <c r="H42" s="19" t="s">
+        <v>252</v>
+      </c>
+      <c r="I42" s="19"/>
       <c r="J42" s="19"/>
       <c r="K42" s="19" t="s">
-        <v>27</v>
+        <v>253</v>
       </c>
       <c r="L42" s="21" t="n">
         <f aca="false">COUNTIF('Fight card'!$I$6:$I$200,A42)+COUNTIF('Fight card'!$K$6:$K$200,A42)</f>
@@ -4977,30 +4865,28 @@
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="20" t="str">
         <f aca="false">TRIM(B43&amp;" "&amp;C43)</f>
-        <v>Ambre BEAUVOIR</v>
+        <v>YVAN BOYER</v>
       </c>
       <c r="B43" s="19" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="C43" s="19" t="s">
-        <v>260</v>
+        <v>198</v>
       </c>
       <c r="D43" s="19" t="s">
-        <v>261</v>
+        <v>220</v>
       </c>
       <c r="E43" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D43,Clubs!$A$2:$A$20,0)),"")</f>
-        <v>SHO</v>
+        <v>MAN</v>
       </c>
       <c r="F43" s="19" t="s">
-        <v>176</v>
-      </c>
-      <c r="G43" s="19" t="s">
-        <v>181</v>
-      </c>
+        <v>161</v>
+      </c>
+      <c r="G43" s="19"/>
       <c r="H43" s="19"/>
       <c r="I43" s="19" t="n">
-        <v>59</v>
+        <v>40</v>
       </c>
       <c r="J43" s="19"/>
       <c r="K43" s="19" t="s">
@@ -5015,108 +4901,106 @@
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="20" t="str">
         <f aca="false">TRIM(B44&amp;" "&amp;C44)</f>
-        <v>Chloé FONTAINE</v>
+        <v>Ambre BEAUVOIR</v>
       </c>
       <c r="B44" s="19" t="s">
-        <v>262</v>
+        <v>255</v>
       </c>
       <c r="C44" s="19" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D44" s="19" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
       <c r="E44" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D44,Clubs!$A$2:$A$20,0)),"")</f>
         <v>SHO</v>
       </c>
       <c r="F44" s="19" t="s">
+        <v>171</v>
+      </c>
+      <c r="G44" s="19" t="s">
         <v>176</v>
       </c>
-      <c r="G44" s="19"/>
       <c r="H44" s="19"/>
       <c r="I44" s="19" t="n">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="J44" s="19"/>
       <c r="K44" s="19" t="s">
-        <v>45</v>
+        <v>27</v>
       </c>
       <c r="L44" s="21" t="n">
         <f aca="false">COUNTIF('Fight card'!$I$6:$I$200,A44)+COUNTIF('Fight card'!$K$6:$K$200,A44)</f>
         <v>1</v>
       </c>
-      <c r="M44" s="19" t="s">
-        <v>263</v>
-      </c>
+      <c r="M44" s="19"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="20" t="str">
         <f aca="false">TRIM(B45&amp;" "&amp;C45)</f>
-        <v>Emmanuelle GRUCHET</v>
+        <v>Chloé FONTAINE</v>
       </c>
       <c r="B45" s="19" t="s">
-        <v>264</v>
+        <v>258</v>
       </c>
       <c r="C45" s="19" t="s">
-        <v>265</v>
+        <v>251</v>
       </c>
       <c r="D45" s="19" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
       <c r="E45" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D45,Clubs!$A$2:$A$20,0)),"")</f>
         <v>SHO</v>
       </c>
       <c r="F45" s="19" t="s">
-        <v>176</v>
-      </c>
-      <c r="G45" s="19" t="s">
-        <v>181</v>
-      </c>
+        <v>171</v>
+      </c>
+      <c r="G45" s="19"/>
       <c r="H45" s="19"/>
       <c r="I45" s="19" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="J45" s="19"/>
       <c r="K45" s="19" t="s">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="L45" s="21" t="n">
         <f aca="false">COUNTIF('Fight card'!$I$6:$I$200,A45)+COUNTIF('Fight card'!$K$6:$K$200,A45)</f>
         <v>1</v>
       </c>
-      <c r="M45" s="19"/>
+      <c r="M45" s="19" t="s">
+        <v>259</v>
+      </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="20" t="str">
         <f aca="false">TRIM(B46&amp;" "&amp;C46)</f>
-        <v>Ethan BEGUE</v>
+        <v>Emmanuelle GRUCHET</v>
       </c>
       <c r="B46" s="19" t="s">
-        <v>163</v>
+        <v>260</v>
       </c>
       <c r="C46" s="19" t="s">
-        <v>241</v>
+        <v>261</v>
       </c>
       <c r="D46" s="19" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
       <c r="E46" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D46,Clubs!$A$2:$A$20,0)),"")</f>
         <v>SHO</v>
       </c>
       <c r="F46" s="19" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="G46" s="19" t="s">
-        <v>173</v>
-      </c>
-      <c r="H46" s="19" t="s">
-        <v>266</v>
-      </c>
+        <v>176</v>
+      </c>
+      <c r="H46" s="19"/>
       <c r="I46" s="19" t="n">
-        <v>78</v>
+        <v>55</v>
       </c>
       <c r="J46" s="19"/>
       <c r="K46" s="19" t="s">
@@ -5124,79 +5008,81 @@
       </c>
       <c r="L46" s="21" t="n">
         <f aca="false">COUNTIF('Fight card'!$I$6:$I$200,A46)+COUNTIF('Fight card'!$K$6:$K$200,A46)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M46" s="19"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="20" t="str">
         <f aca="false">TRIM(B47&amp;" "&amp;C47)</f>
-        <v>Jean-Marc SERGE</v>
+        <v>Ethan BEGUE</v>
       </c>
       <c r="B47" s="19" t="s">
-        <v>267</v>
+        <v>159</v>
       </c>
       <c r="C47" s="19" t="s">
-        <v>268</v>
+        <v>237</v>
       </c>
       <c r="D47" s="19" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
       <c r="E47" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D47,Clubs!$A$2:$A$20,0)),"")</f>
         <v>SHO</v>
       </c>
       <c r="F47" s="19" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="G47" s="19" t="s">
-        <v>181</v>
-      </c>
-      <c r="H47" s="19"/>
+        <v>168</v>
+      </c>
+      <c r="H47" s="19" t="s">
+        <v>262</v>
+      </c>
       <c r="I47" s="19" t="n">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="J47" s="19"/>
       <c r="K47" s="19" t="s">
-        <v>99</v>
+        <v>27</v>
       </c>
       <c r="L47" s="21" t="n">
         <f aca="false">COUNTIF('Fight card'!$I$6:$I$200,A47)+COUNTIF('Fight card'!$K$6:$K$200,A47)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M47" s="19"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="20" t="str">
         <f aca="false">TRIM(B48&amp;" "&amp;C48)</f>
-        <v>Lanah BARDINOT</v>
+        <v>Jean-Marc SERGE</v>
       </c>
       <c r="B48" s="19" t="s">
-        <v>269</v>
+        <v>263</v>
       </c>
       <c r="C48" s="19" t="s">
-        <v>270</v>
+        <v>264</v>
       </c>
       <c r="D48" s="19" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
       <c r="E48" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D48,Clubs!$A$2:$A$20,0)),"")</f>
         <v>SHO</v>
       </c>
       <c r="F48" s="19" t="s">
+        <v>161</v>
+      </c>
+      <c r="G48" s="19" t="s">
         <v>176</v>
-      </c>
-      <c r="G48" s="19" t="s">
-        <v>166</v>
       </c>
       <c r="H48" s="19"/>
       <c r="I48" s="19" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="J48" s="19"/>
       <c r="K48" s="19" t="s">
-        <v>27</v>
+        <v>99</v>
       </c>
       <c r="L48" s="21" t="n">
         <f aca="false">COUNTIF('Fight card'!$I$6:$I$200,A48)+COUNTIF('Fight card'!$K$6:$K$200,A48)</f>
@@ -5207,32 +5093,34 @@
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="20" t="str">
         <f aca="false">TRIM(B49&amp;" "&amp;C49)</f>
-        <v>Mathéo GABRIEL</v>
+        <v>Lanah BARDINOT</v>
       </c>
       <c r="B49" s="19" t="s">
-        <v>271</v>
+        <v>265</v>
       </c>
       <c r="C49" s="19" t="s">
-        <v>272</v>
+        <v>266</v>
       </c>
       <c r="D49" s="19" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
       <c r="E49" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D49,Clubs!$A$2:$A$20,0)),"")</f>
         <v>SHO</v>
       </c>
       <c r="F49" s="19" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="G49" s="19" t="s">
-        <v>181</v>
+        <v>162</v>
       </c>
       <c r="H49" s="19"/>
-      <c r="I49" s="19"/>
+      <c r="I49" s="19" t="n">
+        <v>64</v>
+      </c>
       <c r="J49" s="19"/>
       <c r="K49" s="19" t="s">
-        <v>99</v>
+        <v>27</v>
       </c>
       <c r="L49" s="21" t="n">
         <f aca="false">COUNTIF('Fight card'!$I$6:$I$200,A49)+COUNTIF('Fight card'!$K$6:$K$200,A49)</f>
@@ -5243,31 +5131,29 @@
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="20" t="str">
         <f aca="false">TRIM(B50&amp;" "&amp;C50)</f>
-        <v>Miguel IBAO</v>
+        <v>Mathéo GABRIEL</v>
       </c>
       <c r="B50" s="19" t="s">
-        <v>273</v>
+        <v>267</v>
       </c>
       <c r="C50" s="19" t="s">
-        <v>274</v>
+        <v>268</v>
       </c>
       <c r="D50" s="19" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
       <c r="E50" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D50,Clubs!$A$2:$A$20,0)),"")</f>
         <v>SHO</v>
       </c>
       <c r="F50" s="19" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="G50" s="19" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="H50" s="19"/>
-      <c r="I50" s="19" t="n">
-        <v>74</v>
-      </c>
+      <c r="I50" s="19"/>
       <c r="J50" s="19"/>
       <c r="K50" s="19" t="s">
         <v>99</v>
@@ -5281,46 +5167,84 @@
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="20" t="str">
         <f aca="false">TRIM(B51&amp;" "&amp;C51)</f>
-        <v>Thomas GUICHARD</v>
+        <v>Miguel IBAO</v>
       </c>
       <c r="B51" s="19" t="s">
-        <v>275</v>
+        <v>269</v>
       </c>
       <c r="C51" s="19" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
       <c r="D51" s="19" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
       <c r="E51" s="20" t="str">
         <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D51,Clubs!$A$2:$A$20,0)),"")</f>
         <v>SHO</v>
       </c>
       <c r="F51" s="19" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="G51" s="19" t="s">
-        <v>181</v>
-      </c>
-      <c r="H51" s="19" t="s">
-        <v>277</v>
-      </c>
+        <v>176</v>
+      </c>
+      <c r="H51" s="19"/>
       <c r="I51" s="19" t="n">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="J51" s="19"/>
       <c r="K51" s="19" t="s">
-        <v>27</v>
+        <v>99</v>
       </c>
       <c r="L51" s="21" t="n">
         <f aca="false">COUNTIF('Fight card'!$I$6:$I$200,A51)+COUNTIF('Fight card'!$K$6:$K$200,A51)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M51" s="19"/>
     </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="20" t="str">
+        <f aca="false">TRIM(B52&amp;" "&amp;C52)</f>
+        <v>Thomas GUICHARD</v>
+      </c>
+      <c r="B52" s="19" t="s">
+        <v>271</v>
+      </c>
+      <c r="C52" s="19" t="s">
+        <v>272</v>
+      </c>
+      <c r="D52" s="19" t="s">
+        <v>257</v>
+      </c>
+      <c r="E52" s="20" t="str">
+        <f aca="false">IFERROR(INDEX(Clubs!$B$2:$B$20,MATCH(D52,Clubs!$A$2:$A$20,0)),"")</f>
+        <v>SHO</v>
+      </c>
+      <c r="F52" s="19" t="s">
+        <v>161</v>
+      </c>
+      <c r="G52" s="19" t="s">
+        <v>176</v>
+      </c>
+      <c r="H52" s="19" t="s">
+        <v>273</v>
+      </c>
+      <c r="I52" s="19" t="n">
+        <v>84</v>
+      </c>
+      <c r="J52" s="19"/>
+      <c r="K52" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="L52" s="21" t="n">
+        <f aca="false">COUNTIF('Fight card'!$I$6:$I$200,A52)+COUNTIF('Fight card'!$K$6:$K$200,A52)</f>
+        <v>1</v>
+      </c>
+      <c r="M52" s="19"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M51"/>
-  <conditionalFormatting sqref="L2:L51">
+  <autoFilter ref="A1:M52"/>
+  <conditionalFormatting sqref="L2:L52">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
       <formula>L2=0</formula>
     </cfRule>
@@ -5354,39 +5278,39 @@
         <v>15</v>
       </c>
       <c r="B1" s="18" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="19" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="B2" s="19" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="19" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="B3" s="19" t="s">
-        <v>279</v>
+        <v>275</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="19" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>280</v>
+        <v>276</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="19" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
     </row>
   </sheetData>

</xml_diff>